<commit_message>
Fix PDF export glitches; open model on Cover in Base Case
CIM and teaser (LibreOffice export bugs): sentence-final periods and '?' shown
at line start, number ranges reversed to line end (200-300bps, 12-24, 2023-2024),
stat tiles reversed (8 YRS, ~78%, ~15,000 FT ...), two-digit page badges and
TOC page numbers wrapped digit by digit; TOC renumbered to match page badges.
Model: opens on Cover at top-left, scenario = Base Case (EV 11.0) to match the
teaser/CIM headline; all cached values recalculated (526 formulas verified).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/public/files/ironbend-financial-model.xlsx
+++ b/public/files/ironbend-financial-model.xlsx
@@ -5,7 +5,7 @@
   <workbookPr/>
   <xr:revisionPtr revIDLastSave="0" documentId="8_{8FE06411-AFE7-4EED-B24E-7CB30D459F96}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" activeTab="9" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" activeTab="0" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Cover" sheetId="1" r:id="rId1"/>
@@ -31,7 +31,7 @@
     <definedName name="_xlnm.Print_Area" localSheetId="6">'Sources &amp; Uses'!$A$1:$G$28</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="5">Valuation!$A$1:$G$25</definedName>
   </definedNames>
-  <calcPr calcId="191028" iterateDelta="1E-4"/>
+  <calcPr calcId="191028" iterateDelta="1E-4" fullCalcOnLoad="1"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -1919,7 +1919,7 @@
       </c>
       <c r="C6" s="61">
         <f>'Sources &amp; Uses'!C17</f>
-        <v>4.6800000000000015</v>
+        <v>4.06</v>
       </c>
     </row>
     <row r="7" spans="2:8" ht="15" customHeight="1">
@@ -1928,7 +1928,7 @@
       </c>
       <c r="C7" s="41">
         <f>'Sources &amp; Uses'!C16</f>
-        <v>1.95</v>
+        <v>1.65</v>
       </c>
     </row>
     <row r="8" spans="2:8" ht="15" customHeight="1">
@@ -1937,7 +1937,7 @@
       </c>
       <c r="C8" s="35">
         <f>Assumptions!C51</f>
-        <v>6.5</v>
+        <v>5.5</v>
       </c>
     </row>
     <row r="10" spans="2:8" ht="18" customHeight="1">
@@ -1954,7 +1954,7 @@
       </c>
       <c r="C11" s="41">
         <f>'Income Statement'!L11</f>
-        <v>3.701531291074561</v>
+        <v>3.04678516694153</v>
       </c>
     </row>
     <row r="12" spans="2:8" ht="15" customHeight="1">
@@ -1963,7 +1963,7 @@
       </c>
       <c r="C12" s="35">
         <f>Assumptions!C51</f>
-        <v>6.5</v>
+        <v>5.5</v>
       </c>
     </row>
     <row r="13" spans="2:8" ht="15" customHeight="1">
@@ -1972,7 +1972,7 @@
       </c>
       <c r="C13" s="53">
         <f>C11*C12</f>
-        <v>24.059953391984646</v>
+        <v>16.7573184181784</v>
       </c>
     </row>
     <row r="14" spans="2:8" ht="15" customHeight="1">
@@ -1981,7 +1981,7 @@
       </c>
       <c r="C14" s="41">
         <f>-'Cash Flow &amp; Debt Schedule'!G10</f>
-        <v>-1</v>
+        <v>-0.833333333333333</v>
       </c>
     </row>
     <row r="15" spans="2:8" ht="15" customHeight="1">
@@ -1990,7 +1990,7 @@
       </c>
       <c r="C15" s="41">
         <f>-'Cash Flow &amp; Debt Schedule'!G15</f>
-        <v>-1.3</v>
+        <v>-1.1</v>
       </c>
     </row>
     <row r="16" spans="2:8" ht="15" customHeight="1">
@@ -1999,7 +1999,7 @@
       </c>
       <c r="C16" s="53">
         <f>C13+C14+C15</f>
-        <v>21.759953391984645</v>
+        <v>14.8239850848451</v>
       </c>
     </row>
     <row r="18" spans="2:8" ht="18" customHeight="1">
@@ -2016,7 +2016,7 @@
       </c>
       <c r="C19" s="29">
         <f>C6/(C6+C7)</f>
-        <v>0.70588235294117652</v>
+        <v>0.711033274956217</v>
       </c>
     </row>
     <row r="20" spans="2:8" ht="15" customHeight="1">
@@ -2025,7 +2025,7 @@
       </c>
       <c r="C20" s="53">
         <f>C16*C19</f>
-        <v>15.359967100224456</v>
+        <v>10.5403466627795</v>
       </c>
     </row>
     <row r="22" spans="2:8" ht="15" customHeight="1">
@@ -2034,7 +2034,7 @@
       </c>
       <c r="C22" s="58">
         <f>C20/C6</f>
-        <v>3.2820442521847117</v>
+        <v>2.59614449822156</v>
       </c>
     </row>
     <row r="23" spans="2:8" ht="15" customHeight="1">
@@ -2051,7 +2051,7 @@
       </c>
       <c r="C24" s="72">
         <f>IRR(C28:H28)</f>
-        <v>0.2683201332598486</v>
+        <v>0.210224030728596</v>
       </c>
     </row>
     <row r="26" spans="2:8" ht="18" customHeight="1">
@@ -2094,7 +2094,7 @@
       </c>
       <c r="C28" s="30">
         <f>-C6</f>
-        <v>-4.6800000000000015</v>
+        <v>-4.06</v>
       </c>
       <c r="D28" s="30">
         <v>0</v>
@@ -2110,7 +2110,7 @@
       </c>
       <c r="H28" s="30">
         <f>C20</f>
-        <v>15.359967100224456</v>
+        <v>10.5403466627795</v>
       </c>
     </row>
     <row r="30" spans="2:8" ht="27.75" customHeight="1">
@@ -2267,7 +2267,7 @@
         <v>50</v>
       </c>
       <c r="C13" s="4" t="s">
-        <v>51</v>
+        <v>54</v>
       </c>
       <c r="D13" s="4"/>
     </row>
@@ -2353,7 +2353,7 @@
       </c>
       <c r="C22" s="24">
         <f>INDEX(C16:E16,MATCH(C13,$C$15:$E$15,0))</f>
-        <v>0.08</v>
+        <v>0.055</v>
       </c>
     </row>
     <row r="23" spans="2:6" ht="15" customHeight="1">
@@ -2362,7 +2362,7 @@
       </c>
       <c r="C23" s="25">
         <f>INDEX(C17:E17,MATCH(C13,$C$15:$E$15,0))</f>
-        <v>90</v>
+        <v>50</v>
       </c>
     </row>
     <row r="24" spans="2:6" ht="15" customHeight="1">
@@ -2371,7 +2371,7 @@
       </c>
       <c r="C24" s="26">
         <f>INDEX(C18:E18,MATCH(C13,$C$15:$E$15,0))</f>
-        <v>6.5</v>
+        <v>5.5</v>
       </c>
     </row>
     <row r="25" spans="2:6" ht="15" customHeight="1">
@@ -2380,7 +2380,7 @@
       </c>
       <c r="C25" s="26">
         <f>INDEX(C19:E19,MATCH(C13,$C$15:$E$15,0))</f>
-        <v>3</v>
+        <v>2.5</v>
       </c>
     </row>
     <row r="27" spans="2:6" ht="18.75" customHeight="1">
@@ -2431,7 +2431,7 @@
       </c>
       <c r="F31" s="30">
         <f>C31*E31</f>
-        <v>1.1015999999999999</v>
+        <v>1.1016</v>
       </c>
     </row>
     <row r="32" spans="2:6" ht="15" customHeight="1">
@@ -2443,14 +2443,14 @@
       </c>
       <c r="D32" s="29">
         <f>C32/C31-1</f>
-        <v>0.11764705882352944</v>
+        <v>0.117647058823529</v>
       </c>
       <c r="E32" s="21">
         <v>0.17799999999999999</v>
       </c>
       <c r="F32" s="30">
         <f>C32*E32</f>
-        <v>1.3527999999999998</v>
+        <v>1.3528</v>
       </c>
     </row>
     <row r="33" spans="2:6" ht="15" customHeight="1">
@@ -2462,14 +2462,14 @@
       </c>
       <c r="D33" s="29">
         <f>C33/C32-1</f>
-        <v>9.2105263157894912E-2</v>
+        <v>0.0921052631578949</v>
       </c>
       <c r="E33" s="21">
         <v>0.193</v>
       </c>
       <c r="F33" s="30">
         <f>C33*E33</f>
-        <v>1.6019000000000001</v>
+        <v>1.6019</v>
       </c>
     </row>
     <row r="34" spans="2:6" ht="15" customHeight="1">
@@ -2481,7 +2481,7 @@
       </c>
       <c r="D34" s="29">
         <f>C34/C33-1</f>
-        <v>7.2289156626506035E-2</v>
+        <v>0.072289156626506</v>
       </c>
       <c r="E34" s="21">
         <v>0.20799999999999999</v>
@@ -2500,14 +2500,14 @@
       </c>
       <c r="D35" s="29">
         <f>C35/C34-1</f>
-        <v>5.6179775280898792E-2</v>
+        <v>0.0561797752808988</v>
       </c>
       <c r="E35" s="21">
         <v>0.223</v>
       </c>
       <c r="F35" s="30">
         <f>C35*E35</f>
-        <v>2.0962000000000001</v>
+        <v>2.0962</v>
       </c>
     </row>
     <row r="36" spans="2:6" ht="15" customHeight="1">
@@ -2516,7 +2516,7 @@
       </c>
       <c r="C36" s="31">
         <f>(C35/C31)^(1/4)-1</f>
-        <v>8.4313176252373667E-2</v>
+        <v>0.0843131762523737</v>
       </c>
     </row>
     <row r="39" spans="2:6" ht="18" customHeight="1">
@@ -2594,7 +2594,7 @@
       </c>
       <c r="C47" s="33">
         <f>C46/C35</f>
-        <v>0.21276595744680851</v>
+        <v>0.212765957446809</v>
       </c>
     </row>
     <row r="50" spans="2:6" ht="18" customHeight="1">
@@ -2612,7 +2612,7 @@
       </c>
       <c r="C51" s="34">
         <f>C24</f>
-        <v>6.5</v>
+        <v>5.5</v>
       </c>
     </row>
     <row r="52" spans="2:6" ht="15" customHeight="1">
@@ -2656,7 +2656,7 @@
       </c>
       <c r="C57" s="34">
         <f>C25</f>
-        <v>3</v>
+        <v>2.5</v>
       </c>
     </row>
     <row r="58" spans="2:6" ht="15" customHeight="1">
@@ -3038,7 +3038,7 @@
       </c>
       <c r="E6" s="41">
         <f>Assumptions!C33</f>
-        <v>8.3000000000000007</v>
+        <v>8.3</v>
       </c>
       <c r="F6" s="41">
         <f>Assumptions!C34</f>
@@ -3050,23 +3050,23 @@
       </c>
       <c r="H6" s="42">
         <f>G6*(1+Assumptions!C22)</f>
-        <v>10.152000000000001</v>
+        <v>9.917</v>
       </c>
       <c r="I6" s="42">
         <f>H6*(1+Assumptions!C22)</f>
-        <v>10.964160000000001</v>
+        <v>10.462435</v>
       </c>
       <c r="J6" s="42">
         <f>I6*(1+Assumptions!C22)</f>
-        <v>11.841292800000002</v>
+        <v>11.037868925</v>
       </c>
       <c r="K6" s="42">
         <f>J6*(1+Assumptions!C22)</f>
-        <v>12.788596224000003</v>
+        <v>11.644951715875</v>
       </c>
       <c r="L6" s="42">
         <f>K6*(1+Assumptions!C22)</f>
-        <v>13.811683921920004</v>
+        <v>12.2854240602481</v>
       </c>
     </row>
     <row r="7" spans="2:12" ht="15" customHeight="1">
@@ -3075,39 +3075,39 @@
       </c>
       <c r="D7" s="29">
         <f>D6/C6-1</f>
-        <v>0.11764705882352944</v>
+        <v>0.117647058823529</v>
       </c>
       <c r="E7" s="29">
         <f>E6/D6-1</f>
-        <v>9.2105263157894912E-2</v>
+        <v>0.0921052631578949</v>
       </c>
       <c r="F7" s="29">
         <f>F6/E6-1</f>
-        <v>7.2289156626506035E-2</v>
+        <v>0.072289156626506</v>
       </c>
       <c r="G7" s="29">
         <f>G6/F6-1</f>
-        <v>5.6179775280898792E-2</v>
+        <v>0.0561797752808988</v>
       </c>
       <c r="H7" s="43">
         <f>H6/G6-1</f>
-        <v>8.0000000000000071E-2</v>
+        <v>0.0549999999999999</v>
       </c>
       <c r="I7" s="43">
         <f>I6/H6-1</f>
-        <v>8.0000000000000071E-2</v>
+        <v>0.0549999999999999</v>
       </c>
       <c r="J7" s="43">
         <f>J6/I6-1</f>
-        <v>8.0000000000000071E-2</v>
+        <v>0.0549999999999999</v>
       </c>
       <c r="K7" s="43">
         <f>K6/J6-1</f>
-        <v>8.0000000000000071E-2</v>
+        <v>0.0549999999999999</v>
       </c>
       <c r="L7" s="43">
         <f>L6/K6-1</f>
-        <v>8.0000000000000071E-2</v>
+        <v>0.0549999999999999</v>
       </c>
     </row>
     <row r="8" spans="2:12" ht="15" customHeight="1">
@@ -3165,39 +3165,39 @@
       </c>
       <c r="D9" s="46">
         <f>D6*D8</f>
-        <v>2.8119999999999998</v>
+        <v>2.812</v>
       </c>
       <c r="E9" s="46">
         <f>E6*E8</f>
-        <v>3.0710000000000002</v>
+        <v>3.071</v>
       </c>
       <c r="F9" s="46">
         <f>F6*F8</f>
-        <v>3.2930000000000001</v>
+        <v>3.293</v>
       </c>
       <c r="G9" s="46">
         <f>G6*G8</f>
-        <v>3.4780000000000002</v>
+        <v>3.478</v>
       </c>
       <c r="H9" s="42">
         <f>H6*H8</f>
-        <v>3.7562400000000005</v>
+        <v>3.66929</v>
       </c>
       <c r="I9" s="42">
         <f>I6*I8</f>
-        <v>4.0567392000000009</v>
+        <v>3.87110095</v>
       </c>
       <c r="J9" s="42">
         <f>J6*J8</f>
-        <v>4.3812783360000003</v>
+        <v>4.08401150225</v>
       </c>
       <c r="K9" s="42">
         <f>K6*K8</f>
-        <v>4.7317806028800007</v>
+        <v>4.30863213487375</v>
       </c>
       <c r="L9" s="42">
         <f>L6*L8</f>
-        <v>5.1103230511104014</v>
+        <v>4.54560690229181</v>
       </c>
     </row>
     <row r="10" spans="2:12" ht="15" customHeight="1">
@@ -3206,11 +3206,11 @@
       </c>
       <c r="C10" s="44">
         <f>Assumptions!E31</f>
-        <v>0.16200000000000001</v>
+        <v>0.162</v>
       </c>
       <c r="D10" s="44">
         <f>Assumptions!E32</f>
-        <v>0.17799999999999999</v>
+        <v>0.178</v>
       </c>
       <c r="E10" s="44">
         <f>Assumptions!E33</f>
@@ -3218,7 +3218,7 @@
       </c>
       <c r="F10" s="44">
         <f>Assumptions!E34</f>
-        <v>0.20799999999999999</v>
+        <v>0.208</v>
       </c>
       <c r="G10" s="44">
         <f>Assumptions!E35</f>
@@ -3226,23 +3226,23 @@
       </c>
       <c r="H10" s="43">
         <f>G10+Assumptions!C23/10000</f>
-        <v>0.23200000000000001</v>
+        <v>0.228</v>
       </c>
       <c r="I10" s="43">
         <f>H10+Assumptions!C23/10000</f>
-        <v>0.24100000000000002</v>
+        <v>0.233</v>
       </c>
       <c r="J10" s="43">
         <f>I10+Assumptions!C23/10000</f>
-        <v>0.25</v>
+        <v>0.238</v>
       </c>
       <c r="K10" s="43">
         <f>J10+Assumptions!C23/10000</f>
-        <v>0.25900000000000001</v>
+        <v>0.243</v>
       </c>
       <c r="L10" s="43">
         <f>K10+Assumptions!C23/10000</f>
-        <v>0.26800000000000002</v>
+        <v>0.248</v>
       </c>
     </row>
     <row r="11" spans="2:12" ht="15" customHeight="1">
@@ -3251,15 +3251,15 @@
       </c>
       <c r="C11" s="32">
         <f>C6*C10</f>
-        <v>1.1015999999999999</v>
+        <v>1.1016</v>
       </c>
       <c r="D11" s="32">
         <f>D6*D10</f>
-        <v>1.3527999999999998</v>
+        <v>1.3528</v>
       </c>
       <c r="E11" s="32">
         <f>E6*E10</f>
-        <v>1.6019000000000001</v>
+        <v>1.6019</v>
       </c>
       <c r="F11" s="32">
         <f>F6*F10</f>
@@ -3267,27 +3267,27 @@
       </c>
       <c r="G11" s="32">
         <f>G6*G10</f>
-        <v>2.0962000000000001</v>
+        <v>2.0962</v>
       </c>
       <c r="H11" s="47">
         <f>H6*H10</f>
-        <v>2.3552640000000005</v>
+        <v>2.261076</v>
       </c>
       <c r="I11" s="47">
         <f>I6*I10</f>
-        <v>2.6423625600000005</v>
+        <v>2.437747355</v>
       </c>
       <c r="J11" s="47">
         <f>J6*J10</f>
-        <v>2.9603232000000004</v>
+        <v>2.62701280415</v>
       </c>
       <c r="K11" s="47">
         <f>K6*K10</f>
-        <v>3.3122464220160008</v>
+        <v>2.82972326695762</v>
       </c>
       <c r="L11" s="47">
         <f>L6*L10</f>
-        <v>3.701531291074561</v>
+        <v>3.04678516694153</v>
       </c>
     </row>
     <row r="12" spans="2:12" ht="15" customHeight="1">
@@ -3296,43 +3296,43 @@
       </c>
       <c r="C12" s="30">
         <f>C9-C11</f>
-        <v>1.4144000000000001</v>
+        <v>1.4144</v>
       </c>
       <c r="D12" s="30">
         <f>D9-D11</f>
-        <v>1.4592000000000001</v>
+        <v>1.4592</v>
       </c>
       <c r="E12" s="30">
         <f>E9-E11</f>
-        <v>1.4691000000000001</v>
+        <v>1.4691</v>
       </c>
       <c r="F12" s="30">
         <f>F9-F11</f>
-        <v>1.4418000000000002</v>
+        <v>1.4418</v>
       </c>
       <c r="G12" s="30">
         <f>G9-G11</f>
-        <v>1.3818000000000001</v>
+        <v>1.3818</v>
       </c>
       <c r="H12" s="48">
         <f>H9-H11</f>
-        <v>1.400976</v>
+        <v>1.408214</v>
       </c>
       <c r="I12" s="48">
         <f>I9-I11</f>
-        <v>1.4143766400000004</v>
+        <v>1.433353595</v>
       </c>
       <c r="J12" s="48">
         <f>J9-J11</f>
-        <v>1.4209551359999999</v>
+        <v>1.4569986981</v>
       </c>
       <c r="K12" s="48">
         <f>K9-K11</f>
-        <v>1.4195341808639999</v>
+        <v>1.47890886791612</v>
       </c>
       <c r="L12" s="48">
         <f>L9-L11</f>
-        <v>1.4087917600358404</v>
+        <v>1.49882173535027</v>
       </c>
     </row>
     <row r="13" spans="2:12" ht="15" customHeight="1">
@@ -3341,11 +3341,11 @@
       </c>
       <c r="C13" s="30">
         <f>C6*Assumptions!C64</f>
-        <v>0.20399999999999999</v>
+        <v>0.204</v>
       </c>
       <c r="D13" s="30">
         <f>D6*Assumptions!C64</f>
-        <v>0.22799999999999998</v>
+        <v>0.228</v>
       </c>
       <c r="E13" s="30">
         <f>E6*Assumptions!C64</f>
@@ -3353,31 +3353,31 @@
       </c>
       <c r="F13" s="30">
         <f>F6*Assumptions!C64</f>
-        <v>0.26700000000000002</v>
+        <v>0.267</v>
       </c>
       <c r="G13" s="30">
         <f>G6*Assumptions!C64</f>
-        <v>0.28199999999999997</v>
+        <v>0.282</v>
       </c>
       <c r="H13" s="48">
         <f>H6*Assumptions!C64</f>
-        <v>0.30456</v>
+        <v>0.29751</v>
       </c>
       <c r="I13" s="48">
         <f>I6*Assumptions!C64</f>
-        <v>0.32892480000000002</v>
+        <v>0.31387305</v>
       </c>
       <c r="J13" s="48">
         <f>J6*Assumptions!C64</f>
-        <v>0.35523878400000003</v>
+        <v>0.33113606775</v>
       </c>
       <c r="K13" s="48">
         <f>K6*Assumptions!C64</f>
-        <v>0.38365788672000006</v>
+        <v>0.34934855147625</v>
       </c>
       <c r="L13" s="48">
         <f>L6*Assumptions!C64</f>
-        <v>0.41435051765760011</v>
+        <v>0.368562721807444</v>
       </c>
     </row>
     <row r="14" spans="2:12" ht="15" customHeight="1">
@@ -3386,11 +3386,11 @@
       </c>
       <c r="C14" s="32">
         <f>C11-C13</f>
-        <v>0.89759999999999995</v>
+        <v>0.8976</v>
       </c>
       <c r="D14" s="32">
         <f>D11-D13</f>
-        <v>1.1247999999999998</v>
+        <v>1.1248</v>
       </c>
       <c r="E14" s="32">
         <f>E11-E13</f>
@@ -3398,7 +3398,7 @@
       </c>
       <c r="F14" s="32">
         <f>F11-F13</f>
-        <v>1.5842000000000001</v>
+        <v>1.5842</v>
       </c>
       <c r="G14" s="32">
         <f>G11-G13</f>
@@ -3406,23 +3406,23 @@
       </c>
       <c r="H14" s="47">
         <f>H11-H13</f>
-        <v>2.0507040000000005</v>
+        <v>1.963566</v>
       </c>
       <c r="I14" s="47">
         <f>I11-I13</f>
-        <v>2.3134377600000002</v>
+        <v>2.123874305</v>
       </c>
       <c r="J14" s="47">
         <f>J11-J13</f>
-        <v>2.6050844160000004</v>
+        <v>2.2958767364</v>
       </c>
       <c r="K14" s="47">
         <f>K11-K13</f>
-        <v>2.9285885352960008</v>
+        <v>2.48037471548137</v>
       </c>
       <c r="L14" s="47">
         <f>L11-L13</f>
-        <v>3.2871807734169609</v>
+        <v>2.67822244513409</v>
       </c>
     </row>
     <row r="15" spans="2:12" ht="15" customHeight="1">
@@ -3446,23 +3446,23 @@
       </c>
       <c r="H15" s="50">
         <f>'Cash Flow &amp; Debt Schedule'!C17</f>
-        <v>0.62899999999999989</v>
+        <v>0.5255</v>
       </c>
       <c r="I15" s="50">
         <f>'Cash Flow &amp; Debt Schedule'!D17</f>
-        <v>0.54149999999999998</v>
+        <v>0.452583333333333</v>
       </c>
       <c r="J15" s="50">
         <f>'Cash Flow &amp; Debt Schedule'!E17</f>
-        <v>0.45399999999999996</v>
+        <v>0.379666666666667</v>
       </c>
       <c r="K15" s="50">
         <f>'Cash Flow &amp; Debt Schedule'!F17</f>
-        <v>0.36649999999999994</v>
+        <v>0.30675</v>
       </c>
       <c r="L15" s="50">
         <f>'Cash Flow &amp; Debt Schedule'!G17</f>
-        <v>0.27900000000000003</v>
+        <v>0.233833333333333</v>
       </c>
     </row>
     <row r="16" spans="2:12" ht="15" customHeight="1">
@@ -3486,23 +3486,23 @@
       </c>
       <c r="H16" s="47">
         <f>H14-H15</f>
-        <v>1.4217040000000005</v>
+        <v>1.438066</v>
       </c>
       <c r="I16" s="47">
         <f>I14-I15</f>
-        <v>1.7719377600000001</v>
+        <v>1.67129097166667</v>
       </c>
       <c r="J16" s="47">
         <f>J14-J15</f>
-        <v>2.1510844160000007</v>
+        <v>1.91621006973333</v>
       </c>
       <c r="K16" s="47">
         <f>K14-K15</f>
-        <v>2.562088535296001</v>
+        <v>2.17362471548137</v>
       </c>
       <c r="L16" s="47">
         <f>L14-L15</f>
-        <v>3.008180773416961</v>
+        <v>2.44438911180076</v>
       </c>
     </row>
     <row r="17" spans="2:12" ht="15" customHeight="1">
@@ -3526,23 +3526,23 @@
       </c>
       <c r="H17" s="48">
         <f>MAX(H16,0)*Assumptions!C71</f>
-        <v>0.35542600000000013</v>
+        <v>0.3595165</v>
       </c>
       <c r="I17" s="48">
         <f>MAX(I16,0)*Assumptions!C71</f>
-        <v>0.44298444000000003</v>
+        <v>0.417822742916667</v>
       </c>
       <c r="J17" s="48">
         <f>MAX(J16,0)*Assumptions!C71</f>
-        <v>0.53777110400000017</v>
+        <v>0.479052517433333</v>
       </c>
       <c r="K17" s="48">
         <f>MAX(K16,0)*Assumptions!C71</f>
-        <v>0.64052213382400025</v>
+        <v>0.543406178870344</v>
       </c>
       <c r="L17" s="48">
         <f>MAX(L16,0)*Assumptions!C71</f>
-        <v>0.75204519335424025</v>
+        <v>0.61109727795019</v>
       </c>
     </row>
     <row r="18" spans="2:12" ht="15" customHeight="1">
@@ -3566,23 +3566,23 @@
       </c>
       <c r="H18" s="51">
         <f>H16-H17</f>
-        <v>1.0662780000000005</v>
+        <v>1.0785495</v>
       </c>
       <c r="I18" s="51">
         <f>I16-I17</f>
-        <v>1.3289533200000001</v>
+        <v>1.25346822875</v>
       </c>
       <c r="J18" s="51">
         <f>J16-J17</f>
-        <v>1.6133133120000005</v>
+        <v>1.4371575523</v>
       </c>
       <c r="K18" s="51">
         <f>K16-K17</f>
-        <v>1.9215664014720009</v>
+        <v>1.63021853661103</v>
       </c>
       <c r="L18" s="51">
         <f>L16-L17</f>
-        <v>2.256135580062721</v>
+        <v>1.83329183385057</v>
       </c>
     </row>
     <row r="20" spans="2:12" ht="27.75" customHeight="1">
@@ -3692,23 +3692,23 @@
       </c>
       <c r="D7" s="41">
         <f>'Cash Flow &amp; Debt Schedule'!C35</f>
-        <v>0.36808280000000021</v>
+        <v>0.575831966666667</v>
       </c>
       <c r="E7" s="41">
         <f>'Cash Flow &amp; Debt Schedule'!D35</f>
-        <v>0.69898530400000025</v>
+        <v>1.02826653108333</v>
       </c>
       <c r="F7" s="41">
         <f>'Cash Flow &amp; Debt Schedule'!E35</f>
-        <v>1.3144037347200006</v>
+        <v>1.666166900845</v>
       </c>
       <c r="G7" s="41">
         <f>'Cash Flow &amp; Debt Schedule'!F35</f>
-        <v>2.2382436644096009</v>
+        <v>2.49900244321142</v>
       </c>
       <c r="H7" s="41">
         <f>'Cash Flow &amp; Debt Schedule'!G35</f>
-        <v>3.4968346549473295</v>
+        <v>3.53688855146726</v>
       </c>
     </row>
     <row r="8" spans="2:8" ht="15" customHeight="1">
@@ -3717,27 +3717,27 @@
       </c>
       <c r="C8" s="30">
         <f>'Income Statement'!G6*Assumptions!C66</f>
-        <v>1.1279999999999999</v>
+        <v>1.128</v>
       </c>
       <c r="D8" s="30">
         <f>'Income Statement'!H6*Assumptions!C66</f>
-        <v>1.21824</v>
+        <v>1.19004</v>
       </c>
       <c r="E8" s="30">
         <f>'Income Statement'!I6*Assumptions!C66</f>
-        <v>1.3156992000000001</v>
+        <v>1.2554922</v>
       </c>
       <c r="F8" s="30">
         <f>'Income Statement'!J6*Assumptions!C66</f>
-        <v>1.4209551360000001</v>
+        <v>1.324544271</v>
       </c>
       <c r="G8" s="30">
         <f>'Income Statement'!K6*Assumptions!C66</f>
-        <v>1.5346315468800003</v>
+        <v>1.397394205905</v>
       </c>
       <c r="H8" s="30">
         <f>'Income Statement'!L6*Assumptions!C66</f>
-        <v>1.6574020706304005</v>
+        <v>1.47425088722977</v>
       </c>
     </row>
     <row r="9" spans="2:8" ht="15" customHeight="1">
@@ -3746,27 +3746,27 @@
       </c>
       <c r="C9" s="30">
         <f>('Income Statement'!G6-'Income Statement'!G9)*Assumptions!C67</f>
-        <v>0.59220000000000006</v>
+        <v>0.5922</v>
       </c>
       <c r="D9" s="30">
         <f>('Income Statement'!H6-'Income Statement'!H9)*Assumptions!C67</f>
-        <v>0.63957600000000014</v>
+        <v>0.624771</v>
       </c>
       <c r="E9" s="30">
         <f>('Income Statement'!I6-'Income Statement'!I9)*Assumptions!C67</f>
-        <v>0.69074208000000015</v>
+        <v>0.659133405</v>
       </c>
       <c r="F9" s="30">
         <f>('Income Statement'!J6-'Income Statement'!J9)*Assumptions!C67</f>
-        <v>0.74600144640000021</v>
+        <v>0.695385742275</v>
       </c>
       <c r="G9" s="30">
         <f>('Income Statement'!K6-'Income Statement'!K9)*Assumptions!C67</f>
-        <v>0.80568156211200026</v>
+        <v>0.733631958100125</v>
       </c>
       <c r="H9" s="30">
         <f>('Income Statement'!L6-'Income Statement'!L9)*Assumptions!C67</f>
-        <v>0.87013608708096024</v>
+        <v>0.773981715795632</v>
       </c>
     </row>
     <row r="10" spans="2:8" ht="15" customHeight="1">
@@ -3779,23 +3779,23 @@
       </c>
       <c r="D10" s="30">
         <f>C10-'Cash Flow &amp; Debt Schedule'!C27-'Cash Flow &amp; Debt Schedule'!C21</f>
-        <v>2.71848</v>
+        <v>2.72083</v>
       </c>
       <c r="E10" s="30">
         <f>D10-'Cash Flow &amp; Debt Schedule'!D27-'Cash Flow &amp; Debt Schedule'!D21</f>
-        <v>2.6088383999999998</v>
+        <v>2.61620565</v>
       </c>
       <c r="F10" s="30">
         <f>E10-'Cash Flow &amp; Debt Schedule'!E27-'Cash Flow &amp; Debt Schedule'!E21</f>
-        <v>2.4904254719999996</v>
+        <v>2.50582696075</v>
       </c>
       <c r="G10" s="30">
         <f>F10-'Cash Flow &amp; Debt Schedule'!F27-'Cash Flow &amp; Debt Schedule'!F21</f>
-        <v>2.3625395097599995</v>
+        <v>2.38937744359125</v>
       </c>
       <c r="H10" s="30">
         <f>G10-'Cash Flow &amp; Debt Schedule'!G27-'Cash Flow &amp; Debt Schedule'!G21</f>
-        <v>2.2244226705407995</v>
+        <v>2.26652320298877</v>
       </c>
     </row>
     <row r="11" spans="2:8" ht="15" customHeight="1">
@@ -3804,27 +3804,27 @@
       </c>
       <c r="C11" s="30">
         <f>(C15+'Sources &amp; Uses'!C10)-C7-C8-C9-C10</f>
-        <v>9.5635600000000007</v>
+        <v>7.44356</v>
       </c>
       <c r="D11" s="30">
         <f>C11</f>
-        <v>9.5635600000000007</v>
+        <v>7.44356</v>
       </c>
       <c r="E11" s="30">
         <f>D11</f>
-        <v>9.5635600000000007</v>
+        <v>7.44356</v>
       </c>
       <c r="F11" s="30">
         <f>E11</f>
-        <v>9.5635600000000007</v>
+        <v>7.44356</v>
       </c>
       <c r="G11" s="30">
         <f>F11</f>
-        <v>9.5635600000000007</v>
+        <v>7.44356</v>
       </c>
       <c r="H11" s="30">
         <f>G11</f>
-        <v>9.5635600000000007</v>
+        <v>7.44356</v>
       </c>
     </row>
     <row r="12" spans="2:8" ht="15" customHeight="1">
@@ -3833,27 +3833,27 @@
       </c>
       <c r="C12" s="52">
         <f>SUM(C7:C11)</f>
-        <v>14.40376</v>
+        <v>12.28376</v>
       </c>
       <c r="D12" s="52">
         <f>SUM(D7:D11)</f>
-        <v>14.507938800000002</v>
+        <v>12.5550329666667</v>
       </c>
       <c r="E12" s="52">
         <f>SUM(E7:E11)</f>
-        <v>14.877824984</v>
+        <v>13.0026577860833</v>
       </c>
       <c r="F12" s="52">
         <f>SUM(F7:F11)</f>
-        <v>15.535345789120001</v>
+        <v>13.63548387487</v>
       </c>
       <c r="G12" s="52">
         <f>SUM(G7:G11)</f>
-        <v>16.504656283161601</v>
+        <v>14.4629660508078</v>
       </c>
       <c r="H12" s="52">
         <f>SUM(H7:H11)</f>
-        <v>17.812355483199489</v>
+        <v>15.4952043574814</v>
       </c>
     </row>
     <row r="14" spans="2:8" ht="18" customHeight="1">
@@ -3872,27 +3872,27 @@
       </c>
       <c r="C15" s="30">
         <f>('Income Statement'!G6-'Income Statement'!G9)*Assumptions!C68</f>
-        <v>0.47376000000000007</v>
+        <v>0.47376</v>
       </c>
       <c r="D15" s="30">
         <f>('Income Statement'!H6-'Income Statement'!H9)*Assumptions!C68</f>
-        <v>0.51166080000000014</v>
+        <v>0.4998168</v>
       </c>
       <c r="E15" s="30">
         <f>('Income Statement'!I6-'Income Statement'!I9)*Assumptions!C68</f>
-        <v>0.5525936640000001</v>
+        <v>0.527306724</v>
       </c>
       <c r="F15" s="30">
         <f>('Income Statement'!J6-'Income Statement'!J9)*Assumptions!C68</f>
-        <v>0.59680115712000015</v>
+        <v>0.55630859382</v>
       </c>
       <c r="G15" s="30">
         <f>('Income Statement'!K6-'Income Statement'!K9)*Assumptions!C68</f>
-        <v>0.64454524968960014</v>
+        <v>0.5869055664801</v>
       </c>
       <c r="H15" s="30">
         <f>('Income Statement'!L6-'Income Statement'!L9)*Assumptions!C68</f>
-        <v>0.69610886966476815</v>
+        <v>0.619185372636505</v>
       </c>
     </row>
     <row r="16" spans="2:8" ht="15" customHeight="1">
@@ -3901,27 +3901,27 @@
       </c>
       <c r="C16" s="41">
         <f>'Sources &amp; Uses'!C14</f>
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="D16" s="41">
         <f>'Cash Flow &amp; Debt Schedule'!C10</f>
-        <v>5</v>
+        <v>4.16666666666667</v>
       </c>
       <c r="E16" s="41">
         <f>'Cash Flow &amp; Debt Schedule'!D10</f>
-        <v>4</v>
+        <v>3.33333333333333</v>
       </c>
       <c r="F16" s="41">
         <f>'Cash Flow &amp; Debt Schedule'!E10</f>
-        <v>3</v>
+        <v>2.5</v>
       </c>
       <c r="G16" s="41">
         <f>'Cash Flow &amp; Debt Schedule'!F10</f>
-        <v>2</v>
+        <v>1.66666666666667</v>
       </c>
       <c r="H16" s="41">
         <f>'Cash Flow &amp; Debt Schedule'!G10</f>
-        <v>1</v>
+        <v>0.833333333333333</v>
       </c>
     </row>
     <row r="17" spans="2:8" ht="15" customHeight="1">
@@ -3930,27 +3930,27 @@
       </c>
       <c r="C17" s="41">
         <f>'Sources &amp; Uses'!C15</f>
-        <v>1.3</v>
+        <v>1.1</v>
       </c>
       <c r="D17" s="41">
         <f>'Cash Flow &amp; Debt Schedule'!C15</f>
-        <v>1.3</v>
+        <v>1.1</v>
       </c>
       <c r="E17" s="41">
         <f>'Cash Flow &amp; Debt Schedule'!D15</f>
-        <v>1.3</v>
+        <v>1.1</v>
       </c>
       <c r="F17" s="41">
         <f>'Cash Flow &amp; Debt Schedule'!E15</f>
-        <v>1.3</v>
+        <v>1.1</v>
       </c>
       <c r="G17" s="41">
         <f>'Cash Flow &amp; Debt Schedule'!F15</f>
-        <v>1.3</v>
+        <v>1.1</v>
       </c>
       <c r="H17" s="41">
         <f>'Cash Flow &amp; Debt Schedule'!G15</f>
-        <v>1.3</v>
+        <v>1.1</v>
       </c>
     </row>
     <row r="18" spans="2:8" ht="15" customHeight="1">
@@ -3959,27 +3959,27 @@
       </c>
       <c r="C18" s="32">
         <f>SUM(C15:C17)</f>
-        <v>7.7737600000000002</v>
+        <v>6.57376</v>
       </c>
       <c r="D18" s="32">
         <f>SUM(D15:D17)</f>
-        <v>6.8116608000000003</v>
+        <v>5.76648346666667</v>
       </c>
       <c r="E18" s="32">
         <f>SUM(E15:E17)</f>
-        <v>5.8525936639999996</v>
+        <v>4.96064005733333</v>
       </c>
       <c r="F18" s="32">
         <f>SUM(F15:F17)</f>
-        <v>4.8968011571200005</v>
+        <v>4.15630859382</v>
       </c>
       <c r="G18" s="32">
         <f>SUM(G15:G17)</f>
-        <v>3.9445452496896003</v>
+        <v>3.35357223314677</v>
       </c>
       <c r="H18" s="32">
         <f>SUM(H15:H17)</f>
-        <v>2.9961088696647682</v>
+        <v>2.55251870596984</v>
       </c>
     </row>
     <row r="20" spans="2:8" ht="18" customHeight="1">
@@ -3998,27 +3998,27 @@
       </c>
       <c r="C21" s="41">
         <f>'Sources &amp; Uses'!C17</f>
-        <v>4.6800000000000015</v>
+        <v>4.06</v>
       </c>
       <c r="D21" s="41">
         <f>'Sources &amp; Uses'!C17</f>
-        <v>4.6800000000000015</v>
+        <v>4.06</v>
       </c>
       <c r="E21" s="41">
         <f>'Sources &amp; Uses'!C17</f>
-        <v>4.6800000000000015</v>
+        <v>4.06</v>
       </c>
       <c r="F21" s="41">
         <f>'Sources &amp; Uses'!C17</f>
-        <v>4.6800000000000015</v>
+        <v>4.06</v>
       </c>
       <c r="G21" s="41">
         <f>'Sources &amp; Uses'!C17</f>
-        <v>4.6800000000000015</v>
+        <v>4.06</v>
       </c>
       <c r="H21" s="41">
         <f>'Sources &amp; Uses'!C17</f>
-        <v>4.6800000000000015</v>
+        <v>4.06</v>
       </c>
     </row>
     <row r="22" spans="2:8" ht="15" customHeight="1">
@@ -4027,27 +4027,27 @@
       </c>
       <c r="C22" s="41">
         <f>'Sources &amp; Uses'!C16</f>
-        <v>1.95</v>
+        <v>1.65</v>
       </c>
       <c r="D22" s="41">
         <f>'Sources &amp; Uses'!C16</f>
-        <v>1.95</v>
+        <v>1.65</v>
       </c>
       <c r="E22" s="41">
         <f>'Sources &amp; Uses'!C16</f>
-        <v>1.95</v>
+        <v>1.65</v>
       </c>
       <c r="F22" s="41">
         <f>'Sources &amp; Uses'!C16</f>
-        <v>1.95</v>
+        <v>1.65</v>
       </c>
       <c r="G22" s="41">
         <f>'Sources &amp; Uses'!C16</f>
-        <v>1.95</v>
+        <v>1.65</v>
       </c>
       <c r="H22" s="41">
         <f>'Sources &amp; Uses'!C16</f>
-        <v>1.95</v>
+        <v>1.65</v>
       </c>
     </row>
     <row r="23" spans="2:8" ht="15" customHeight="1">
@@ -4059,23 +4059,23 @@
       </c>
       <c r="D23" s="30">
         <f>C23+'Income Statement'!H18</f>
-        <v>1.0662780000000005</v>
+        <v>1.0785495</v>
       </c>
       <c r="E23" s="30">
         <f>D23+'Income Statement'!I18</f>
-        <v>2.3952313200000006</v>
+        <v>2.33201772875</v>
       </c>
       <c r="F23" s="30">
         <f>E23+'Income Statement'!J18</f>
-        <v>4.0085446320000013</v>
+        <v>3.76917528105</v>
       </c>
       <c r="G23" s="30">
         <f>F23+'Income Statement'!K18</f>
-        <v>5.9301110334720022</v>
+        <v>5.39939381766103</v>
       </c>
       <c r="H23" s="30">
         <f>G23+'Income Statement'!L18</f>
-        <v>8.186246613534724</v>
+        <v>7.2326856515116</v>
       </c>
     </row>
     <row r="24" spans="2:8" ht="15" customHeight="1">
@@ -4084,27 +4084,27 @@
       </c>
       <c r="C24" s="32">
         <f>SUM(C21:C23)</f>
-        <v>6.6300000000000017</v>
+        <v>5.71</v>
       </c>
       <c r="D24" s="32">
         <f>SUM(D21:D23)</f>
-        <v>7.6962780000000022</v>
+        <v>6.7885495</v>
       </c>
       <c r="E24" s="32">
         <f>SUM(E21:E23)</f>
-        <v>9.0252313200000032</v>
+        <v>8.04201772875</v>
       </c>
       <c r="F24" s="32">
         <f>SUM(F21:F23)</f>
-        <v>10.638544632000002</v>
+        <v>9.47917528105</v>
       </c>
       <c r="G24" s="32">
         <f>SUM(G21:G23)</f>
-        <v>12.560111033472005</v>
+        <v>11.109393817661</v>
       </c>
       <c r="H24" s="32">
         <f>SUM(H21:H23)</f>
-        <v>14.816246613534727</v>
+        <v>12.9426856515116</v>
       </c>
     </row>
     <row r="26" spans="2:8" ht="15" customHeight="1">
@@ -4113,27 +4113,27 @@
       </c>
       <c r="C26" s="52">
         <f>C18+C24</f>
-        <v>14.403760000000002</v>
+        <v>12.28376</v>
       </c>
       <c r="D26" s="52">
         <f>D18+D24</f>
-        <v>14.507938800000002</v>
+        <v>12.5550329666667</v>
       </c>
       <c r="E26" s="52">
         <f>E18+E24</f>
-        <v>14.877824984000004</v>
+        <v>13.0026577860833</v>
       </c>
       <c r="F26" s="52">
         <f>F18+F24</f>
-        <v>15.535345789120003</v>
+        <v>13.63548387487</v>
       </c>
       <c r="G26" s="52">
         <f>G18+G24</f>
-        <v>16.504656283161605</v>
+        <v>14.4629660508078</v>
       </c>
       <c r="H26" s="52">
         <f>H18+H24</f>
-        <v>17.812355483199497</v>
+        <v>15.4952043574814</v>
       </c>
     </row>
     <row r="27" spans="2:8" ht="15" customHeight="1">
@@ -4262,23 +4262,23 @@
       </c>
       <c r="C7" s="41">
         <f>'Sources &amp; Uses'!C14</f>
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="D7" s="30">
         <f>C10</f>
-        <v>5</v>
+        <v>4.16666666666667</v>
       </c>
       <c r="E7" s="30">
         <f>D10</f>
-        <v>4</v>
+        <v>3.33333333333333</v>
       </c>
       <c r="F7" s="30">
         <f>E10</f>
-        <v>3</v>
+        <v>2.5</v>
       </c>
       <c r="G7" s="30">
         <f>F10</f>
-        <v>2</v>
+        <v>1.66666666666667</v>
       </c>
     </row>
     <row r="8" spans="2:7" ht="15" customHeight="1">
@@ -4287,23 +4287,23 @@
       </c>
       <c r="C8" s="30">
         <f>-MIN(C7, $C$7/Assumptions!C75)</f>
-        <v>-1</v>
+        <v>-0.833333333333333</v>
       </c>
       <c r="D8" s="30">
         <f>-MIN(D7, $C$7/Assumptions!C75)</f>
-        <v>-1</v>
+        <v>-0.833333333333333</v>
       </c>
       <c r="E8" s="30">
         <f>-MIN(E7, $C$7/Assumptions!C75)</f>
-        <v>-1</v>
+        <v>-0.833333333333333</v>
       </c>
       <c r="F8" s="30">
         <f>-MIN(F7, $C$7/Assumptions!C75)</f>
-        <v>-1</v>
+        <v>-0.833333333333333</v>
       </c>
       <c r="G8" s="30">
         <f>-MIN(G7, $C$7/Assumptions!C75)</f>
-        <v>-1</v>
+        <v>-0.833333333333333</v>
       </c>
     </row>
     <row r="9" spans="2:7" ht="15" customHeight="1">
@@ -4312,23 +4312,23 @@
       </c>
       <c r="C9" s="30">
         <f>C7*Assumptions!C74</f>
-        <v>0.52499999999999991</v>
+        <v>0.4375</v>
       </c>
       <c r="D9" s="30">
         <f>D7*Assumptions!C74</f>
-        <v>0.4375</v>
+        <v>0.364583333333333</v>
       </c>
       <c r="E9" s="30">
         <f>E7*Assumptions!C74</f>
-        <v>0.35</v>
+        <v>0.291666666666667</v>
       </c>
       <c r="F9" s="30">
         <f>F7*Assumptions!C74</f>
-        <v>0.26249999999999996</v>
+        <v>0.21875</v>
       </c>
       <c r="G9" s="30">
         <f>G7*Assumptions!C74</f>
-        <v>0.17499999999999999</v>
+        <v>0.145833333333333</v>
       </c>
     </row>
     <row r="10" spans="2:7" ht="15" customHeight="1">
@@ -4337,23 +4337,23 @@
       </c>
       <c r="C10" s="32">
         <f>C7+C8</f>
-        <v>5</v>
+        <v>4.16666666666667</v>
       </c>
       <c r="D10" s="32">
         <f>D7+D8</f>
-        <v>4</v>
+        <v>3.33333333333333</v>
       </c>
       <c r="E10" s="32">
         <f>E7+E8</f>
-        <v>3</v>
+        <v>2.5</v>
       </c>
       <c r="F10" s="32">
         <f>F7+F8</f>
-        <v>2</v>
+        <v>1.66666666666667</v>
       </c>
       <c r="G10" s="32">
         <f>G7+G8</f>
-        <v>1</v>
+        <v>0.833333333333333</v>
       </c>
     </row>
     <row r="12" spans="2:7" ht="18" customHeight="1">
@@ -4372,23 +4372,23 @@
       </c>
       <c r="C13" s="41">
         <f>'Sources &amp; Uses'!C15</f>
-        <v>1.3</v>
+        <v>1.1</v>
       </c>
       <c r="D13" s="30">
         <f>C15</f>
-        <v>1.3</v>
+        <v>1.1</v>
       </c>
       <c r="E13" s="30">
         <f>D15</f>
-        <v>1.3</v>
+        <v>1.1</v>
       </c>
       <c r="F13" s="30">
         <f>E15</f>
-        <v>1.3</v>
+        <v>1.1</v>
       </c>
       <c r="G13" s="30">
         <f>F15</f>
-        <v>1.3</v>
+        <v>1.1</v>
       </c>
     </row>
     <row r="14" spans="2:7" ht="15" customHeight="1">
@@ -4397,23 +4397,23 @@
       </c>
       <c r="C14" s="30">
         <f>C13*Assumptions!C76</f>
-        <v>0.10400000000000001</v>
+        <v>0.088</v>
       </c>
       <c r="D14" s="30">
         <f>D13*Assumptions!C76</f>
-        <v>0.10400000000000001</v>
+        <v>0.088</v>
       </c>
       <c r="E14" s="30">
         <f>E13*Assumptions!C76</f>
-        <v>0.10400000000000001</v>
+        <v>0.088</v>
       </c>
       <c r="F14" s="30">
         <f>F13*Assumptions!C76</f>
-        <v>0.10400000000000001</v>
+        <v>0.088</v>
       </c>
       <c r="G14" s="30">
         <f>G13*Assumptions!C76</f>
-        <v>0.10400000000000001</v>
+        <v>0.088</v>
       </c>
     </row>
     <row r="15" spans="2:7" ht="15" customHeight="1">
@@ -4422,23 +4422,23 @@
       </c>
       <c r="C15" s="32">
         <f>C13</f>
-        <v>1.3</v>
+        <v>1.1</v>
       </c>
       <c r="D15" s="32">
         <f>D13</f>
-        <v>1.3</v>
+        <v>1.1</v>
       </c>
       <c r="E15" s="32">
         <f>E13</f>
-        <v>1.3</v>
+        <v>1.1</v>
       </c>
       <c r="F15" s="32">
         <f>F13</f>
-        <v>1.3</v>
+        <v>1.1</v>
       </c>
       <c r="G15" s="32">
         <f>G13</f>
-        <v>1.3</v>
+        <v>1.1</v>
       </c>
     </row>
     <row r="17" spans="2:7" ht="15" customHeight="1">
@@ -4447,23 +4447,23 @@
       </c>
       <c r="C17" s="53">
         <f>C9+C14</f>
-        <v>0.62899999999999989</v>
+        <v>0.5255</v>
       </c>
       <c r="D17" s="53">
         <f>D9+D14</f>
-        <v>0.54149999999999998</v>
+        <v>0.452583333333333</v>
       </c>
       <c r="E17" s="53">
         <f>E9+E14</f>
-        <v>0.45399999999999996</v>
+        <v>0.379666666666667</v>
       </c>
       <c r="F17" s="53">
         <f>F9+F14</f>
-        <v>0.36649999999999994</v>
+        <v>0.30675</v>
       </c>
       <c r="G17" s="53">
         <f>G9+G14</f>
-        <v>0.27900000000000003</v>
+        <v>0.233833333333333</v>
       </c>
     </row>
     <row r="19" spans="2:7" ht="18" customHeight="1">
@@ -4482,23 +4482,23 @@
       </c>
       <c r="C20" s="41">
         <f>'Income Statement'!H18</f>
-        <v>1.0662780000000005</v>
+        <v>1.0785495</v>
       </c>
       <c r="D20" s="41">
         <f>'Income Statement'!I18</f>
-        <v>1.3289533200000001</v>
+        <v>1.25346822875</v>
       </c>
       <c r="E20" s="41">
         <f>'Income Statement'!J18</f>
-        <v>1.6133133120000005</v>
+        <v>1.4371575523</v>
       </c>
       <c r="F20" s="41">
         <f>'Income Statement'!K18</f>
-        <v>1.9215664014720009</v>
+        <v>1.63021853661103</v>
       </c>
       <c r="G20" s="41">
         <f>'Income Statement'!L18</f>
-        <v>2.256135580062721</v>
+        <v>1.83329183385057</v>
       </c>
     </row>
     <row r="21" spans="2:7" ht="15" customHeight="1">
@@ -4507,23 +4507,23 @@
       </c>
       <c r="C21" s="41">
         <f>'Income Statement'!H13</f>
-        <v>0.30456</v>
+        <v>0.29751</v>
       </c>
       <c r="D21" s="41">
         <f>'Income Statement'!I13</f>
-        <v>0.32892480000000002</v>
+        <v>0.31387305</v>
       </c>
       <c r="E21" s="41">
         <f>'Income Statement'!J13</f>
-        <v>0.35523878400000003</v>
+        <v>0.33113606775</v>
       </c>
       <c r="F21" s="41">
         <f>'Income Statement'!K13</f>
-        <v>0.38365788672000006</v>
+        <v>0.34934855147625</v>
       </c>
       <c r="G21" s="41">
         <f>'Income Statement'!L13</f>
-        <v>0.41435051765760011</v>
+        <v>0.368562721807444</v>
       </c>
     </row>
     <row r="22" spans="2:7" ht="15" customHeight="1">
@@ -4532,23 +4532,23 @@
       </c>
       <c r="C22" s="30">
         <f>-('Balance Sheet'!D8-'Balance Sheet'!C8)</f>
-        <v>-9.0240000000000098E-2</v>
+        <v>-0.0620400000000001</v>
       </c>
       <c r="D22" s="30">
         <f>-('Balance Sheet'!E8-'Balance Sheet'!D8)</f>
-        <v>-9.7459200000000079E-2</v>
+        <v>-0.0654522</v>
       </c>
       <c r="E22" s="30">
         <f>-('Balance Sheet'!F8-'Balance Sheet'!E8)</f>
-        <v>-0.10525593600000005</v>
+        <v>-0.0690520709999998</v>
       </c>
       <c r="F22" s="30">
         <f>-('Balance Sheet'!G8-'Balance Sheet'!F8)</f>
-        <v>-0.11367641088000013</v>
+        <v>-0.0728499349049998</v>
       </c>
       <c r="G22" s="30">
         <f>-('Balance Sheet'!H8-'Balance Sheet'!G8)</f>
-        <v>-0.12277052375040021</v>
+        <v>-0.0768566813247751</v>
       </c>
     </row>
     <row r="23" spans="2:7" ht="15" customHeight="1">
@@ -4557,23 +4557,23 @@
       </c>
       <c r="C23" s="30">
         <f>-('Balance Sheet'!D9-'Balance Sheet'!C9)</f>
-        <v>-4.7376000000000085E-2</v>
+        <v>-0.0325709999999999</v>
       </c>
       <c r="D23" s="30">
         <f>-('Balance Sheet'!E9-'Balance Sheet'!D9)</f>
-        <v>-5.1166080000000003E-2</v>
+        <v>-0.034362405</v>
       </c>
       <c r="E23" s="30">
         <f>-('Balance Sheet'!F9-'Balance Sheet'!E9)</f>
-        <v>-5.5259366400000065E-2</v>
+        <v>-0.036252337275</v>
       </c>
       <c r="F23" s="30">
         <f>-('Balance Sheet'!G9-'Balance Sheet'!F9)</f>
-        <v>-5.9680115712000048E-2</v>
+        <v>-0.038246215825125</v>
       </c>
       <c r="G23" s="30">
         <f>-('Balance Sheet'!H9-'Balance Sheet'!G9)</f>
-        <v>-6.4454524968959981E-2</v>
+        <v>-0.0403497576955068</v>
       </c>
     </row>
     <row r="24" spans="2:7" ht="15" customHeight="1">
@@ -4582,23 +4582,23 @@
       </c>
       <c r="C24" s="30">
         <f>('Balance Sheet'!D15-'Balance Sheet'!C15)</f>
-        <v>3.7900800000000068E-2</v>
+        <v>0.0260567999999999</v>
       </c>
       <c r="D24" s="30">
         <f>('Balance Sheet'!E15-'Balance Sheet'!D15)</f>
-        <v>4.0932863999999958E-2</v>
+        <v>0.027489924</v>
       </c>
       <c r="E24" s="30">
         <f>('Balance Sheet'!F15-'Balance Sheet'!E15)</f>
-        <v>4.4207493120000052E-2</v>
+        <v>0.0290018698199999</v>
       </c>
       <c r="F24" s="30">
         <f>('Balance Sheet'!G15-'Balance Sheet'!F15)</f>
-        <v>4.7744092569599994E-2</v>
+        <v>0.0305969726601</v>
       </c>
       <c r="G24" s="30">
         <f>('Balance Sheet'!H15-'Balance Sheet'!G15)</f>
-        <v>5.1563619975168007E-2</v>
+        <v>0.0322798061564056</v>
       </c>
     </row>
     <row r="25" spans="2:7" ht="15" customHeight="1">
@@ -4607,23 +4607,23 @@
       </c>
       <c r="C25" s="32">
         <f>SUM(C20:C24)</f>
-        <v>1.2711228000000003</v>
+        <v>1.3075053</v>
       </c>
       <c r="D25" s="32">
         <f>SUM(D20:D24)</f>
-        <v>1.550185704</v>
+        <v>1.49501659775</v>
       </c>
       <c r="E25" s="32">
         <f>SUM(E20:E24)</f>
-        <v>1.8522442867200004</v>
+        <v>1.691991081595</v>
       </c>
       <c r="F25" s="32">
         <f>SUM(F20:F24)</f>
-        <v>2.1796118541696003</v>
+        <v>1.89906791001726</v>
       </c>
       <c r="G25" s="32">
         <f>SUM(G20:G24)</f>
-        <v>2.5348246689761287</v>
+        <v>2.11692792279414</v>
       </c>
     </row>
     <row r="27" spans="2:7" ht="15" customHeight="1">
@@ -4632,23 +4632,23 @@
       </c>
       <c r="C27" s="30">
         <f>-'Income Statement'!H6*Assumptions!C65</f>
-        <v>-0.20304000000000003</v>
+        <v>-0.19834</v>
       </c>
       <c r="D27" s="30">
         <f>-'Income Statement'!I6*Assumptions!C65</f>
-        <v>-0.21928320000000004</v>
+        <v>-0.2092487</v>
       </c>
       <c r="E27" s="30">
         <f>-'Income Statement'!J6*Assumptions!C65</f>
-        <v>-0.23682585600000003</v>
+        <v>-0.2207573785</v>
       </c>
       <c r="F27" s="30">
         <f>-'Income Statement'!K6*Assumptions!C65</f>
-        <v>-0.25577192448000008</v>
+        <v>-0.2328990343175</v>
       </c>
       <c r="G27" s="30">
         <f>-'Income Statement'!L6*Assumptions!C65</f>
-        <v>-0.27623367843840008</v>
+        <v>-0.245708481204962</v>
       </c>
     </row>
     <row r="28" spans="2:7" ht="15" customHeight="1">
@@ -4657,23 +4657,23 @@
       </c>
       <c r="C28" s="32">
         <f>C27</f>
-        <v>-0.20304000000000003</v>
+        <v>-0.19834</v>
       </c>
       <c r="D28" s="32">
         <f>D27</f>
-        <v>-0.21928320000000004</v>
+        <v>-0.2092487</v>
       </c>
       <c r="E28" s="32">
         <f>E27</f>
-        <v>-0.23682585600000003</v>
+        <v>-0.2207573785</v>
       </c>
       <c r="F28" s="32">
         <f>F27</f>
-        <v>-0.25577192448000008</v>
+        <v>-0.2328990343175</v>
       </c>
       <c r="G28" s="32">
         <f>G27</f>
-        <v>-0.27623367843840008</v>
+        <v>-0.245708481204962</v>
       </c>
     </row>
     <row r="30" spans="2:7" ht="15" customHeight="1">
@@ -4682,23 +4682,23 @@
       </c>
       <c r="C30" s="30">
         <f>C8</f>
-        <v>-1</v>
+        <v>-0.833333333333333</v>
       </c>
       <c r="D30" s="30">
         <f>D8</f>
-        <v>-1</v>
+        <v>-0.833333333333333</v>
       </c>
       <c r="E30" s="30">
         <f>E8</f>
-        <v>-1</v>
+        <v>-0.833333333333333</v>
       </c>
       <c r="F30" s="30">
         <f>F8</f>
-        <v>-1</v>
+        <v>-0.833333333333333</v>
       </c>
       <c r="G30" s="30">
         <f>G8</f>
-        <v>-1</v>
+        <v>-0.833333333333333</v>
       </c>
     </row>
     <row r="31" spans="2:7" ht="15" customHeight="1">
@@ -4707,23 +4707,23 @@
       </c>
       <c r="C31" s="32">
         <f>C30</f>
-        <v>-1</v>
+        <v>-0.833333333333333</v>
       </c>
       <c r="D31" s="32">
         <f>D30</f>
-        <v>-1</v>
+        <v>-0.833333333333333</v>
       </c>
       <c r="E31" s="32">
         <f>E30</f>
-        <v>-1</v>
+        <v>-0.833333333333333</v>
       </c>
       <c r="F31" s="32">
         <f>F30</f>
-        <v>-1</v>
+        <v>-0.833333333333333</v>
       </c>
       <c r="G31" s="32">
         <f>G30</f>
-        <v>-1</v>
+        <v>-0.833333333333333</v>
       </c>
     </row>
     <row r="33" spans="2:7" ht="15" customHeight="1">
@@ -4732,23 +4732,23 @@
       </c>
       <c r="C33" s="53">
         <f>C25+C28+C31</f>
-        <v>6.8082800000000221E-2</v>
+        <v>0.275831966666667</v>
       </c>
       <c r="D33" s="53">
         <f>D25+D28+D31</f>
-        <v>0.33090250399999999</v>
+        <v>0.452434564416667</v>
       </c>
       <c r="E33" s="53">
         <f>E25+E28+E31</f>
-        <v>0.61541843072000035</v>
+        <v>0.637900369761666</v>
       </c>
       <c r="F33" s="53">
         <f>F25+F28+F31</f>
-        <v>0.92383992968960027</v>
+        <v>0.832835542366423</v>
       </c>
       <c r="G33" s="53">
         <f>G25+G28+G31</f>
-        <v>1.2585909905377286</v>
+        <v>1.03788610825584</v>
       </c>
     </row>
     <row r="34" spans="2:7" ht="15" customHeight="1">
@@ -4761,19 +4761,19 @@
       </c>
       <c r="D34" s="30">
         <f>C35</f>
-        <v>0.36808280000000021</v>
+        <v>0.575831966666667</v>
       </c>
       <c r="E34" s="30">
         <f>D35</f>
-        <v>0.69898530400000025</v>
+        <v>1.02826653108333</v>
       </c>
       <c r="F34" s="30">
         <f>E35</f>
-        <v>1.3144037347200006</v>
+        <v>1.666166900845</v>
       </c>
       <c r="G34" s="30">
         <f>F35</f>
-        <v>2.2382436644096009</v>
+        <v>2.49900244321142</v>
       </c>
     </row>
     <row r="35" spans="2:7" ht="15" customHeight="1">
@@ -4782,23 +4782,23 @@
       </c>
       <c r="C35" s="52">
         <f>C34+C33</f>
-        <v>0.36808280000000021</v>
+        <v>0.575831966666667</v>
       </c>
       <c r="D35" s="52">
         <f>D34+D33</f>
-        <v>0.69898530400000025</v>
+        <v>1.02826653108333</v>
       </c>
       <c r="E35" s="52">
         <f>E34+E33</f>
-        <v>1.3144037347200006</v>
+        <v>1.666166900845</v>
       </c>
       <c r="F35" s="52">
         <f>F34+F33</f>
-        <v>2.2382436644096009</v>
+        <v>2.49900244321142</v>
       </c>
       <c r="G35" s="52">
         <f>G34+G33</f>
-        <v>3.4968346549473295</v>
+        <v>3.53688855146726</v>
       </c>
     </row>
     <row r="37" spans="2:7" ht="18.75" customHeight="1">
@@ -4885,7 +4885,7 @@
       </c>
       <c r="C7" s="55">
         <f>Assumptions!C51</f>
-        <v>6.5</v>
+        <v>5.5</v>
       </c>
     </row>
     <row r="8" spans="2:6" ht="15" customHeight="1">
@@ -4894,7 +4894,7 @@
       </c>
       <c r="C8" s="53">
         <f>C6*C7</f>
-        <v>13</v>
+        <v>11</v>
       </c>
     </row>
     <row r="9" spans="2:6" ht="15" customHeight="1">
@@ -4903,7 +4903,7 @@
       </c>
       <c r="C9" s="56">
         <f>C8/Assumptions!C35</f>
-        <v>1.3829787234042552</v>
+        <v>1.17021276595745</v>
       </c>
     </row>
     <row r="11" spans="2:6" ht="18" customHeight="1">
@@ -4946,11 +4946,11 @@
       </c>
       <c r="C14" s="58">
         <f>C7</f>
-        <v>6.5</v>
+        <v>5.5</v>
       </c>
       <c r="D14" s="59">
         <f>C8</f>
-        <v>13</v>
+        <v>11</v>
       </c>
     </row>
     <row r="15" spans="2:6" ht="15" customHeight="1">
@@ -4989,7 +4989,7 @@
       </c>
       <c r="C19" s="30">
         <f>C8</f>
-        <v>13</v>
+        <v>11</v>
       </c>
     </row>
     <row r="20" spans="2:5" ht="15" customHeight="1">
@@ -5007,7 +5007,7 @@
       </c>
       <c r="C21" s="53">
         <f>C19+C20</f>
-        <v>13</v>
+        <v>11</v>
       </c>
     </row>
     <row r="23" spans="2:5" ht="18.75" customHeight="1">
@@ -5097,11 +5097,11 @@
       </c>
       <c r="C7" s="41">
         <f>Valuation!C8</f>
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="D7" s="29">
         <f>C7/C10</f>
-        <v>0.93323761665470195</v>
+        <v>0.931414055884843</v>
       </c>
     </row>
     <row r="8" spans="2:6" ht="15" customHeight="1">
@@ -5110,11 +5110,11 @@
       </c>
       <c r="C8" s="41">
         <f>'Advisor Fee'!C18</f>
-        <v>0.8</v>
+        <v>0.7</v>
       </c>
       <c r="D8" s="29">
         <f>C8/C10</f>
-        <v>5.7430007178750894E-2</v>
+        <v>0.0592718035563082</v>
       </c>
     </row>
     <row r="9" spans="2:6" ht="15" customHeight="1">
@@ -5123,11 +5123,11 @@
       </c>
       <c r="C9" s="30">
         <f>Assumptions!C60*C7</f>
-        <v>0.13</v>
+        <v>0.11</v>
       </c>
       <c r="D9" s="29">
         <f>C9/C10</f>
-        <v>9.3323761665470208E-3</v>
+        <v>0.00931414055884843</v>
       </c>
     </row>
     <row r="10" spans="2:6" ht="15" customHeight="1">
@@ -5136,7 +5136,7 @@
       </c>
       <c r="C10" s="53">
         <f>SUM(C7:C9)</f>
-        <v>13.930000000000001</v>
+        <v>11.81</v>
       </c>
     </row>
     <row r="12" spans="2:6" ht="18" customHeight="1">
@@ -5166,11 +5166,11 @@
       </c>
       <c r="C14" s="41">
         <f>Assumptions!C57*Assumptions!C46</f>
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="D14" s="29">
         <f>C14/C18</f>
-        <v>0.4307250538406317</v>
+        <v>0.423370025402202</v>
       </c>
     </row>
     <row r="15" spans="2:6" ht="15" customHeight="1">
@@ -5179,11 +5179,11 @@
       </c>
       <c r="C15" s="41">
         <f>Assumptions!C58*C7</f>
-        <v>1.3</v>
+        <v>1.1</v>
       </c>
       <c r="D15" s="29">
         <f>C15/C18</f>
-        <v>9.3323761665470198E-2</v>
+        <v>0.0931414055884843</v>
       </c>
     </row>
     <row r="16" spans="2:6" ht="15" customHeight="1">
@@ -5192,11 +5192,11 @@
       </c>
       <c r="C16" s="41">
         <f>Assumptions!C59*C7</f>
-        <v>1.95</v>
+        <v>1.65</v>
       </c>
       <c r="D16" s="29">
         <f>C16/C18</f>
-        <v>0.1399856424982053</v>
+        <v>0.139712108382727</v>
       </c>
     </row>
     <row r="17" spans="2:5" ht="15" customHeight="1">
@@ -5205,11 +5205,11 @@
       </c>
       <c r="C17" s="30">
         <f>C10-C14-C15-C16</f>
-        <v>4.6800000000000015</v>
+        <v>4.06</v>
       </c>
       <c r="D17" s="29">
         <f>C17/C18</f>
-        <v>0.33596554199569284</v>
+        <v>0.343776460626588</v>
       </c>
     </row>
     <row r="18" spans="2:5" ht="15" customHeight="1">
@@ -5218,7 +5218,7 @@
       </c>
       <c r="C18" s="53">
         <f>SUM(C14:C17)</f>
-        <v>13.930000000000001</v>
+        <v>11.81</v>
       </c>
     </row>
     <row r="20" spans="2:5" ht="15" customHeight="1">
@@ -5244,7 +5244,7 @@
       </c>
       <c r="C23" s="56">
         <f>C14/Assumptions!C46</f>
-        <v>3</v>
+        <v>2.5</v>
       </c>
     </row>
     <row r="24" spans="2:5" ht="15" customHeight="1">
@@ -5253,7 +5253,7 @@
       </c>
       <c r="C24" s="29">
         <f>C17/C18</f>
-        <v>0.33596554199569284</v>
+        <v>0.343776460626588</v>
       </c>
     </row>
     <row r="25" spans="2:5" ht="15" customHeight="1">
@@ -5332,7 +5332,7 @@
       </c>
       <c r="C5" s="61">
         <f>Valuation!C8</f>
-        <v>13</v>
+        <v>11</v>
       </c>
     </row>
     <row r="7" spans="2:7" ht="18" customHeight="1">
@@ -5380,7 +5380,7 @@
       </c>
       <c r="E9" s="44">
         <f>Assumptions!E81</f>
-        <v>7.0000000000000007E-2</v>
+        <v>0.07</v>
       </c>
       <c r="F9" s="30">
         <f>MIN(MAX(C5-C9,0),D9-C9)</f>
@@ -5388,7 +5388,7 @@
       </c>
       <c r="G9" s="30">
         <f>F9*E9</f>
-        <v>0.35000000000000003</v>
+        <v>0.35</v>
       </c>
     </row>
     <row r="10" spans="2:7" ht="15" customHeight="1">
@@ -5436,11 +5436,11 @@
       </c>
       <c r="F11" s="30">
         <f>MIN(MAX(C5-C11,0),D11-C11)</f>
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="G11" s="30">
         <f>F11*E11</f>
-        <v>0.15000000000000002</v>
+        <v>0.05</v>
       </c>
     </row>
     <row r="12" spans="2:7" ht="15" customHeight="1">
@@ -5508,7 +5508,7 @@
       </c>
       <c r="G14" s="53">
         <f>SUM(G9:G13)</f>
-        <v>0.8</v>
+        <v>0.7</v>
       </c>
     </row>
     <row r="16" spans="2:7" ht="18" customHeight="1">
@@ -5536,7 +5536,7 @@
       </c>
       <c r="C18" s="53">
         <f>MAX(G14,C17)</f>
-        <v>0.8</v>
+        <v>0.7</v>
       </c>
     </row>
     <row r="19" spans="2:7" ht="15" customHeight="1">
@@ -5545,7 +5545,7 @@
       </c>
       <c r="C19" s="65">
         <f>C18/C5</f>
-        <v>6.1538461538461542E-2</v>
+        <v>0.0636363636363636</v>
       </c>
     </row>
     <row r="20" spans="2:7" ht="15" customHeight="1">
@@ -5554,7 +5554,7 @@
       </c>
       <c r="C20" s="66">
         <f>C18*1000000</f>
-        <v>800000</v>
+        <v>700000</v>
       </c>
     </row>
     <row r="22" spans="2:7" ht="27.75" customHeight="1">
@@ -5693,11 +5693,11 @@
       </c>
       <c r="E7" s="30">
         <f>P7</f>
-        <v>0.59000000000000008</v>
+        <v>0.59</v>
       </c>
       <c r="F7" s="65">
         <f>E7/D7</f>
-        <v>6.5555555555555561E-2</v>
+        <v>0.0655555555555556</v>
       </c>
       <c r="G7" s="30">
         <f>D7-Assumptions!C54</f>
@@ -5705,7 +5705,7 @@
       </c>
       <c r="J7" s="30">
         <f>MIN(MAX($D7-Assumptions!$C$81,0),Assumptions!$D$81-Assumptions!$C$81)*Assumptions!$E$81</f>
-        <v>0.35000000000000003</v>
+        <v>0.35</v>
       </c>
       <c r="K7" s="30">
         <f>MIN(MAX($D7-Assumptions!$C$82,0),Assumptions!$D$82-Assumptions!$C$82)*Assumptions!$E$82</f>
@@ -5725,11 +5725,11 @@
       </c>
       <c r="O7" s="30">
         <f>SUM(J7:N7)</f>
-        <v>0.59000000000000008</v>
+        <v>0.59</v>
       </c>
       <c r="P7" s="46">
         <f>MAX(O7,Assumptions!C86)</f>
-        <v>0.59000000000000008</v>
+        <v>0.59</v>
       </c>
     </row>
     <row r="8" spans="2:16" ht="15" customHeight="1">
@@ -5746,11 +5746,11 @@
       </c>
       <c r="E8" s="30">
         <f>P8</f>
-        <v>0.62000000000000011</v>
+        <v>0.62</v>
       </c>
       <c r="F8" s="65">
         <f>E8/D8</f>
-        <v>6.5263157894736856E-2</v>
+        <v>0.0652631578947369</v>
       </c>
       <c r="G8" s="30">
         <f>D8-Assumptions!C54</f>
@@ -5758,7 +5758,7 @@
       </c>
       <c r="J8" s="30">
         <f>MIN(MAX($D8-Assumptions!$C$81,0),Assumptions!$D$81-Assumptions!$C$81)*Assumptions!$E$81</f>
-        <v>0.35000000000000003</v>
+        <v>0.35</v>
       </c>
       <c r="K8" s="30">
         <f>MIN(MAX($D8-Assumptions!$C$82,0),Assumptions!$D$82-Assumptions!$C$82)*Assumptions!$E$82</f>
@@ -5778,11 +5778,11 @@
       </c>
       <c r="O8" s="30">
         <f>SUM(J8:N8)</f>
-        <v>0.62000000000000011</v>
+        <v>0.62</v>
       </c>
       <c r="P8" s="46">
         <f>MAX(O8,Assumptions!C86)</f>
-        <v>0.62000000000000011</v>
+        <v>0.62</v>
       </c>
     </row>
     <row r="9" spans="2:16" ht="15" customHeight="1">
@@ -5803,7 +5803,7 @@
       </c>
       <c r="F9" s="65">
         <f>E9/D9</f>
-        <v>6.5000000000000002E-2</v>
+        <v>0.065</v>
       </c>
       <c r="G9" s="30">
         <f>D9-Assumptions!C54</f>
@@ -5811,7 +5811,7 @@
       </c>
       <c r="J9" s="30">
         <f>MIN(MAX($D9-Assumptions!$C$81,0),Assumptions!$D$81-Assumptions!$C$81)*Assumptions!$E$81</f>
-        <v>0.35000000000000003</v>
+        <v>0.35</v>
       </c>
       <c r="K9" s="30">
         <f>MIN(MAX($D9-Assumptions!$C$82,0),Assumptions!$D$82-Assumptions!$C$82)*Assumptions!$E$82</f>
@@ -5852,11 +5852,11 @@
       </c>
       <c r="E10" s="30">
         <f>P10</f>
-        <v>0.67500000000000004</v>
+        <v>0.675</v>
       </c>
       <c r="F10" s="65">
         <f>E10/D10</f>
-        <v>6.4285714285714293E-2</v>
+        <v>0.0642857142857143</v>
       </c>
       <c r="G10" s="30">
         <f>D10-Assumptions!C54</f>
@@ -5864,7 +5864,7 @@
       </c>
       <c r="J10" s="30">
         <f>MIN(MAX($D10-Assumptions!$C$81,0),Assumptions!$D$81-Assumptions!$C$81)*Assumptions!$E$81</f>
-        <v>0.35000000000000003</v>
+        <v>0.35</v>
       </c>
       <c r="K10" s="30">
         <f>MIN(MAX($D10-Assumptions!$C$82,0),Assumptions!$D$82-Assumptions!$C$82)*Assumptions!$E$82</f>
@@ -5872,7 +5872,7 @@
       </c>
       <c r="L10" s="30">
         <f>MIN(MAX($D10-Assumptions!$C$83,0),Assumptions!$D$83-Assumptions!$C$83)*Assumptions!$E$83</f>
-        <v>2.5000000000000001E-2</v>
+        <v>0.025</v>
       </c>
       <c r="M10" s="30">
         <f>MIN(MAX($D10-Assumptions!$C$84,0),Assumptions!$D$84-Assumptions!$C$84)*Assumptions!$E$84</f>
@@ -5884,11 +5884,11 @@
       </c>
       <c r="O10" s="30">
         <f>SUM(J10:N10)</f>
-        <v>0.67500000000000004</v>
+        <v>0.675</v>
       </c>
       <c r="P10" s="46">
         <f>MAX(O10,Assumptions!C86)</f>
-        <v>0.67500000000000004</v>
+        <v>0.675</v>
       </c>
     </row>
     <row r="11" spans="2:16" ht="15" customHeight="1">
@@ -5905,11 +5905,11 @@
       </c>
       <c r="E11" s="70">
         <f>P11</f>
-        <v>0.70000000000000007</v>
+        <v>0.7</v>
       </c>
       <c r="F11" s="71">
         <f>E11/D11</f>
-        <v>6.3636363636363644E-2</v>
+        <v>0.0636363636363636</v>
       </c>
       <c r="G11" s="70">
         <f>D11-Assumptions!C54</f>
@@ -5917,7 +5917,7 @@
       </c>
       <c r="J11" s="30">
         <f>MIN(MAX($D11-Assumptions!$C$81,0),Assumptions!$D$81-Assumptions!$C$81)*Assumptions!$E$81</f>
-        <v>0.35000000000000003</v>
+        <v>0.35</v>
       </c>
       <c r="K11" s="30">
         <f>MIN(MAX($D11-Assumptions!$C$82,0),Assumptions!$D$82-Assumptions!$C$82)*Assumptions!$E$82</f>
@@ -5937,11 +5937,11 @@
       </c>
       <c r="O11" s="30">
         <f>SUM(J11:N11)</f>
-        <v>0.70000000000000007</v>
+        <v>0.7</v>
       </c>
       <c r="P11" s="46">
         <f>MAX(O11,Assumptions!C86)</f>
-        <v>0.70000000000000007</v>
+        <v>0.7</v>
       </c>
     </row>
     <row r="12" spans="2:16" ht="15" customHeight="1">
@@ -5958,11 +5958,11 @@
       </c>
       <c r="E12" s="30">
         <f>P12</f>
-        <v>0.72500000000000009</v>
+        <v>0.725</v>
       </c>
       <c r="F12" s="65">
         <f>E12/D12</f>
-        <v>6.3043478260869576E-2</v>
+        <v>0.0630434782608696</v>
       </c>
       <c r="G12" s="30">
         <f>D12-Assumptions!C54</f>
@@ -5970,7 +5970,7 @@
       </c>
       <c r="J12" s="30">
         <f>MIN(MAX($D12-Assumptions!$C$81,0),Assumptions!$D$81-Assumptions!$C$81)*Assumptions!$E$81</f>
-        <v>0.35000000000000003</v>
+        <v>0.35</v>
       </c>
       <c r="K12" s="30">
         <f>MIN(MAX($D12-Assumptions!$C$82,0),Assumptions!$D$82-Assumptions!$C$82)*Assumptions!$E$82</f>
@@ -5978,7 +5978,7 @@
       </c>
       <c r="L12" s="30">
         <f>MIN(MAX($D12-Assumptions!$C$83,0),Assumptions!$D$83-Assumptions!$C$83)*Assumptions!$E$83</f>
-        <v>7.5000000000000011E-2</v>
+        <v>0.075</v>
       </c>
       <c r="M12" s="30">
         <f>MIN(MAX($D12-Assumptions!$C$84,0),Assumptions!$D$84-Assumptions!$C$84)*Assumptions!$E$84</f>
@@ -5990,11 +5990,11 @@
       </c>
       <c r="O12" s="30">
         <f>SUM(J12:N12)</f>
-        <v>0.72500000000000009</v>
+        <v>0.725</v>
       </c>
       <c r="P12" s="46">
         <f>MAX(O12,Assumptions!C86)</f>
-        <v>0.72500000000000009</v>
+        <v>0.725</v>
       </c>
     </row>
     <row r="13" spans="2:16" ht="15" customHeight="1">
@@ -6015,7 +6015,7 @@
       </c>
       <c r="F13" s="65">
         <f>E13/D13</f>
-        <v>6.25E-2</v>
+        <v>0.0625</v>
       </c>
       <c r="G13" s="30">
         <f>D13-Assumptions!C54</f>
@@ -6023,7 +6023,7 @@
       </c>
       <c r="J13" s="30">
         <f>MIN(MAX($D13-Assumptions!$C$81,0),Assumptions!$D$81-Assumptions!$C$81)*Assumptions!$E$81</f>
-        <v>0.35000000000000003</v>
+        <v>0.35</v>
       </c>
       <c r="K13" s="30">
         <f>MIN(MAX($D13-Assumptions!$C$82,0),Assumptions!$D$82-Assumptions!$C$82)*Assumptions!$E$82</f>
@@ -6064,11 +6064,11 @@
       </c>
       <c r="E14" s="30">
         <f>P14</f>
-        <v>0.77500000000000002</v>
+        <v>0.775</v>
       </c>
       <c r="F14" s="65">
         <f>E14/D14</f>
-        <v>6.2E-2</v>
+        <v>0.062</v>
       </c>
       <c r="G14" s="30">
         <f>D14-Assumptions!C54</f>
@@ -6076,7 +6076,7 @@
       </c>
       <c r="J14" s="30">
         <f>MIN(MAX($D14-Assumptions!$C$81,0),Assumptions!$D$81-Assumptions!$C$81)*Assumptions!$E$81</f>
-        <v>0.35000000000000003</v>
+        <v>0.35</v>
       </c>
       <c r="K14" s="30">
         <f>MIN(MAX($D14-Assumptions!$C$82,0),Assumptions!$D$82-Assumptions!$C$82)*Assumptions!$E$82</f>
@@ -6096,11 +6096,11 @@
       </c>
       <c r="O14" s="30">
         <f>SUM(J14:N14)</f>
-        <v>0.77500000000000002</v>
+        <v>0.775</v>
       </c>
       <c r="P14" s="46">
         <f>MAX(O14,Assumptions!C86)</f>
-        <v>0.77500000000000002</v>
+        <v>0.775</v>
       </c>
     </row>
     <row r="15" spans="2:16" ht="15" customHeight="1">
@@ -6121,7 +6121,7 @@
       </c>
       <c r="F15" s="65">
         <f>E15/D15</f>
-        <v>6.1538461538461542E-2</v>
+        <v>0.0615384615384615</v>
       </c>
       <c r="G15" s="30">
         <f>D15-Assumptions!C54</f>
@@ -6129,7 +6129,7 @@
       </c>
       <c r="J15" s="30">
         <f>MIN(MAX($D15-Assumptions!$C$81,0),Assumptions!$D$81-Assumptions!$C$81)*Assumptions!$E$81</f>
-        <v>0.35000000000000003</v>
+        <v>0.35</v>
       </c>
       <c r="K15" s="30">
         <f>MIN(MAX($D15-Assumptions!$C$82,0),Assumptions!$D$82-Assumptions!$C$82)*Assumptions!$E$82</f>
@@ -6137,7 +6137,7 @@
       </c>
       <c r="L15" s="30">
         <f>MIN(MAX($D15-Assumptions!$C$83,0),Assumptions!$D$83-Assumptions!$C$83)*Assumptions!$E$83</f>
-        <v>0.15000000000000002</v>
+        <v>0.15</v>
       </c>
       <c r="M15" s="30">
         <f>MIN(MAX($D15-Assumptions!$C$84,0),Assumptions!$D$84-Assumptions!$C$84)*Assumptions!$E$84</f>
@@ -6193,7 +6193,7 @@
       </c>
       <c r="D22" s="30">
         <f>E7</f>
-        <v>0.59000000000000008</v>
+        <v>0.59</v>
       </c>
     </row>
     <row r="23" spans="2:7" ht="15" customHeight="1">

</xml_diff>

<commit_message>
Model: correct CIM page references in labels
Historical financials p.9 -> §IX p.10; EBITDA normalization p.10 -> §X p.11;
valuation cross-check p.16 -> §XVII p.18; gross margin now cites the p.6
segment mix (58% x 34% + 42% x 41% = 37%) instead of a nonexistent p.2 figure.
Labels only; no numbers changed.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/public/files/ironbend-financial-model.xlsx
+++ b/public/files/ironbend-financial-model.xlsx
@@ -286,7 +286,7 @@
     <t>Change 'Selected Scenario' above (dropdown) to Low Case / Base Case / High Case and every downstream tab — Income Statement, Balance Sheet, Cash Flow, Valuation, Sources &amp; Uses, Advisor Fee, and Returns — recalculates automatically.</t>
   </si>
   <si>
-    <t>Historical Financials  (per CIM, p.9)</t>
+    <t>Historical Financials  (per CIM §IX, p.10)</t>
   </si>
   <si>
     <t>Fiscal Year</t>
@@ -322,7 +322,7 @@
     <t>Revenue CAGR (2021 – 2025E)</t>
   </si>
   <si>
-    <t>EBITDA Normalization (2025E)  —  per CIM p.10, management-indicated, preliminary</t>
+    <t>EBITDA Normalization (2025E)  —  per CIM §X, p.11, management-indicated, preliminary</t>
   </si>
   <si>
     <t>Line Item</t>
@@ -385,7 +385,7 @@
     <t>Operating &amp; Balance Sheet Assumptions  (Illustrative — Not Disclosed in CIM)</t>
   </si>
   <si>
-    <t>Gross Margin (held constant; per CIM p.2 disclosed gross margin)</t>
+    <t>Gross Margin (held constant; CIM p.6 segment mix: 58% × 34% + 42% × 41% ≈ 37%)</t>
   </si>
   <si>
     <t>Depreciation &amp; Amortization (% of Revenue)</t>
@@ -679,7 +679,7 @@
     <t>Implied EV / 2025E Revenue</t>
   </si>
   <si>
-    <t>Cross-Check vs. CIM Indicative Range (p.16)</t>
+    <t>Cross-Check vs. CIM Indicative Range (§XVII, p.18)</t>
   </si>
   <si>
     <t>Scenario</t>

</xml_diff>

<commit_message>
Model: keep capex at the CIM's maintenance level (~2% of revenue)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/public/files/ironbend-financial-model.xlsx
+++ b/public/files/ironbend-financial-model.xlsx
@@ -1893,7 +1893,7 @@
       </c>
       <c r="C16" s="41">
         <f>'Cash Flow &amp; Debt Schedule'!G35</f>
-        <v>2.55858887249475</v>
+        <v>3.11206566950598</v>
       </c>
     </row>
     <row r="17" ht="15" customHeight="1" s="12">
@@ -1904,7 +1904,7 @@
       </c>
       <c r="C17" s="53">
         <f>C13+C14+C15+C16</f>
-        <v>16.6910614179487</v>
+        <v>17.2445382149599</v>
       </c>
     </row>
     <row r="18" s="12"/>
@@ -1934,7 +1934,7 @@
       </c>
       <c r="C21" s="53">
         <f>C17*C20</f>
-        <v>11.5045734067217</v>
+        <v>11.8860658882774</v>
       </c>
     </row>
     <row r="22" s="12"/>
@@ -1946,7 +1946,7 @@
       </c>
       <c r="C23" s="58">
         <f>C21/C6</f>
-        <v>3.14332606741029</v>
+        <v>3.24755898586815</v>
       </c>
     </row>
     <row r="24" ht="15" customHeight="1" s="12">
@@ -1967,7 +1967,7 @@
       </c>
       <c r="C25" s="72">
         <f>IRR(C29:H29)</f>
-        <v>0.25741282846414</v>
+        <v>0.265643548200267</v>
       </c>
     </row>
     <row r="26" s="12"/>
@@ -2039,7 +2039,7 @@
       </c>
       <c r="H29" s="30">
         <f>C21</f>
-        <v>11.5045734067217</v>
+        <v>11.8860658882774</v>
       </c>
     </row>
     <row r="30" s="12"/>
@@ -2717,11 +2717,11 @@
     <row r="65" ht="15" customHeight="1" s="12">
       <c r="B65" s="16" t="inlineStr">
         <is>
-          <t>Capital Expenditures (% of Revenue; maintenance ≈ D&amp;A, cf. CIM 2021–22 capex of 2.5–3.1%)</t>
+          <t>Capital Expenditures (% of Revenue)</t>
         </is>
       </c>
       <c r="C65" s="21" t="n">
-        <v>0.03</v>
+        <v>0.02</v>
       </c>
     </row>
     <row r="66" ht="15" customHeight="1" s="12">
@@ -3950,23 +3950,23 @@
       </c>
       <c r="D7" s="41">
         <f>'Cash Flow &amp; Debt Schedule'!C35</f>
-        <v>0.400543716666667</v>
+        <v>0.499713716666667</v>
       </c>
       <c r="E7" s="41">
         <f>'Cash Flow &amp; Debt Schedule'!D35</f>
-        <v>0.668049177333333</v>
+        <v>0.871843527333333</v>
       </c>
       <c r="F7" s="41">
         <f>'Cash Flow &amp; Debt Schedule'!E35</f>
-        <v>1.11084934263875</v>
+        <v>1.42502238188875</v>
       </c>
       <c r="G7" s="41">
         <f>'Cash Flow &amp; Debt Schedule'!F35</f>
-        <v>1.73785416930383</v>
+        <v>2.16847672571258</v>
       </c>
       <c r="H7" s="41">
         <f>'Cash Flow &amp; Debt Schedule'!G35</f>
-        <v>2.55858887249475</v>
+        <v>3.11206566950598</v>
       </c>
     </row>
     <row r="8" ht="15" customHeight="1" s="12">
@@ -4043,23 +4043,23 @@
       </c>
       <c r="D10" s="30">
         <f>C10-'Cash Flow &amp; Debt Schedule'!C27-'Cash Flow &amp; Debt Schedule'!C21</f>
-        <v>2.82</v>
+        <v>2.72083</v>
       </c>
       <c r="E10" s="30">
         <f>D10-'Cash Flow &amp; Debt Schedule'!D27-'Cash Flow &amp; Debt Schedule'!D21</f>
-        <v>2.82</v>
+        <v>2.61620565</v>
       </c>
       <c r="F10" s="30">
         <f>E10-'Cash Flow &amp; Debt Schedule'!E27-'Cash Flow &amp; Debt Schedule'!E21</f>
-        <v>2.82</v>
+        <v>2.50582696075</v>
       </c>
       <c r="G10" s="30">
         <f>F10-'Cash Flow &amp; Debt Schedule'!F27-'Cash Flow &amp; Debt Schedule'!F21</f>
-        <v>2.82</v>
+        <v>2.38937744359125</v>
       </c>
       <c r="H10" s="30">
         <f>G10-'Cash Flow &amp; Debt Schedule'!G27-'Cash Flow &amp; Debt Schedule'!G21</f>
-        <v>2.82</v>
+        <v>2.26652320298877</v>
       </c>
     </row>
     <row r="11" ht="15" customHeight="1" s="12">
@@ -4113,7 +4113,7 @@
       </c>
       <c r="F12" s="52">
         <f>SUM(F7:F11)</f>
-        <v>12.8843393559138</v>
+        <v>12.8843393559137</v>
       </c>
       <c r="G12" s="52">
         <f>SUM(G7:G11)</f>
@@ -4945,23 +4945,23 @@
       </c>
       <c r="C27" s="30">
         <f>-'Income Statement'!H6*Assumptions!C65</f>
-        <v>-0.29751</v>
+        <v>-0.19834</v>
       </c>
       <c r="D27" s="30">
         <f>-'Income Statement'!I6*Assumptions!C65</f>
-        <v>-0.31387305</v>
+        <v>-0.2092487</v>
       </c>
       <c r="E27" s="30">
         <f>-'Income Statement'!J6*Assumptions!C65</f>
-        <v>-0.33113606775</v>
+        <v>-0.2207573785</v>
       </c>
       <c r="F27" s="30">
         <f>-'Income Statement'!K6*Assumptions!C65</f>
-        <v>-0.34934855147625</v>
+        <v>-0.2328990343175</v>
       </c>
       <c r="G27" s="30">
         <f>-'Income Statement'!L6*Assumptions!C65</f>
-        <v>-0.368562721807444</v>
+        <v>-0.245708481204962</v>
       </c>
     </row>
     <row r="28" ht="15" customHeight="1" s="12">
@@ -4972,23 +4972,23 @@
       </c>
       <c r="C28" s="32">
         <f>C27</f>
-        <v>-0.29751</v>
+        <v>-0.19834</v>
       </c>
       <c r="D28" s="32">
         <f>D27</f>
-        <v>-0.31387305</v>
+        <v>-0.2092487</v>
       </c>
       <c r="E28" s="32">
         <f>E27</f>
-        <v>-0.33113606775</v>
+        <v>-0.2207573785</v>
       </c>
       <c r="F28" s="32">
         <f>F27</f>
-        <v>-0.34934855147625</v>
+        <v>-0.2328990343175</v>
       </c>
       <c r="G28" s="32">
         <f>G27</f>
-        <v>-0.368562721807444</v>
+        <v>-0.245708481204962</v>
       </c>
     </row>
     <row r="30" ht="15" customHeight="1" s="12">
@@ -5053,23 +5053,23 @@
       </c>
       <c r="C33" s="53">
         <f>C25+C28+C31</f>
-        <v>0.100543716666667</v>
+        <v>0.199713716666667</v>
       </c>
       <c r="D33" s="53">
         <f>D25+D28+D31</f>
-        <v>0.267505460666667</v>
+        <v>0.372129810666667</v>
       </c>
       <c r="E33" s="53">
         <f>E25+E28+E31</f>
-        <v>0.442800165305416</v>
+        <v>0.553178854555417</v>
       </c>
       <c r="F33" s="53">
         <f>F25+F28+F31</f>
-        <v>0.627004826665079</v>
+        <v>0.743454343823829</v>
       </c>
       <c r="G33" s="53">
         <f>G25+G28+G31</f>
-        <v>0.820734703190922</v>
+        <v>0.943588943793403</v>
       </c>
     </row>
     <row r="34" ht="15" customHeight="1" s="12">
@@ -5084,19 +5084,19 @@
       </c>
       <c r="D34" s="30">
         <f>C35</f>
-        <v>0.400543716666667</v>
+        <v>0.499713716666667</v>
       </c>
       <c r="E34" s="30">
         <f>D35</f>
-        <v>0.668049177333333</v>
+        <v>0.871843527333333</v>
       </c>
       <c r="F34" s="30">
         <f>E35</f>
-        <v>1.11084934263875</v>
+        <v>1.42502238188875</v>
       </c>
       <c r="G34" s="30">
         <f>F35</f>
-        <v>1.73785416930383</v>
+        <v>2.16847672571258</v>
       </c>
     </row>
     <row r="35" ht="15" customHeight="1" s="12">
@@ -5107,23 +5107,23 @@
       </c>
       <c r="C35" s="52">
         <f>C34+C33</f>
-        <v>0.400543716666667</v>
+        <v>0.499713716666667</v>
       </c>
       <c r="D35" s="52">
         <f>D34+D33</f>
-        <v>0.668049177333333</v>
+        <v>0.871843527333333</v>
       </c>
       <c r="E35" s="52">
         <f>E34+E33</f>
-        <v>1.11084934263875</v>
+        <v>1.42502238188875</v>
       </c>
       <c r="F35" s="52">
         <f>F34+F33</f>
-        <v>1.73785416930383</v>
+        <v>2.16847672571258</v>
       </c>
       <c r="G35" s="52">
         <f>G34+G33</f>
-        <v>2.55858887249475</v>
+        <v>3.11206566950598</v>
       </c>
     </row>
     <row r="37" ht="18.75" customHeight="1" s="12">
@@ -5434,15 +5434,15 @@
       </c>
       <c r="C27" s="30">
         <f>MIN(DCF!D56:F58)</f>
-        <v>11.4454948495028</v>
+        <v>12.2351899932778</v>
       </c>
       <c r="D27" s="30">
         <f>MAX(DCF!D56:F58)</f>
-        <v>14.0520914648884</v>
+        <v>15.0173526115104</v>
       </c>
       <c r="E27" s="30">
         <f>AVERAGE(C27:D27)</f>
-        <v>12.7487931571956</v>
+        <v>13.6262713023941</v>
       </c>
     </row>
     <row r="28">
@@ -5453,15 +5453,15 @@
       </c>
       <c r="C28" s="30">
         <f>MIN(DCF!D64:F66)</f>
-        <v>12.2071439265797</v>
+        <v>12.5885268567052</v>
       </c>
       <c r="D28" s="30">
         <f>MAX(DCF!D64:F66)</f>
-        <v>14.5443424170995</v>
+        <v>14.9413878273623</v>
       </c>
       <c r="E28" s="30">
         <f>AVERAGE(C28:D28)</f>
-        <v>13.3757431718396</v>
+        <v>13.7649573420338</v>
       </c>
     </row>
     <row r="29">
@@ -5760,23 +5760,23 @@
       </c>
       <c r="C13" s="41">
         <f>'Cash Flow &amp; Debt Schedule'!C27</f>
-        <v>-0.29751</v>
+        <v>-0.19834</v>
       </c>
       <c r="D13" s="41">
         <f>'Cash Flow &amp; Debt Schedule'!D27</f>
-        <v>-0.31387305</v>
+        <v>-0.2092487</v>
       </c>
       <c r="E13" s="41">
         <f>'Cash Flow &amp; Debt Schedule'!E27</f>
-        <v>-0.33113606775</v>
+        <v>-0.2207573785</v>
       </c>
       <c r="F13" s="41">
         <f>'Cash Flow &amp; Debt Schedule'!F27</f>
-        <v>-0.34934855147625</v>
+        <v>-0.2328990343175</v>
       </c>
       <c r="G13" s="41">
         <f>'Cash Flow &amp; Debt Schedule'!G27</f>
-        <v>-0.368562721807444</v>
+        <v>-0.245708481204962</v>
       </c>
     </row>
     <row r="14">
@@ -5814,23 +5814,23 @@
       </c>
       <c r="C15" s="53">
         <f>SUM(C11:C14)</f>
-        <v>1.32800205</v>
+        <v>1.42717205</v>
       </c>
       <c r="D15" s="53">
         <f>SUM(D11:D14)</f>
-        <v>1.440276294</v>
+        <v>1.544900644</v>
       </c>
       <c r="E15" s="53">
         <f>SUM(E11:E14)</f>
-        <v>1.56088349863875</v>
+        <v>1.67126218788875</v>
       </c>
       <c r="F15" s="53">
         <f>SUM(F11:F14)</f>
-        <v>1.69040065999841</v>
+        <v>1.80685017715716</v>
       </c>
       <c r="G15" s="53">
         <f>SUM(G11:G14)</f>
-        <v>1.82944303652426</v>
+        <v>1.95229727712674</v>
       </c>
     </row>
     <row r="16">
@@ -5841,23 +5841,23 @@
       </c>
       <c r="C16" s="29">
         <f>C15/C7</f>
-        <v>0.614933910913439</v>
+        <v>0.660854770708261</v>
       </c>
       <c r="D16" s="29">
         <f>D15/D7</f>
-        <v>0.617965480248238</v>
+        <v>0.662855642616911</v>
       </c>
       <c r="E16" s="29">
         <f>E15/E7</f>
-        <v>0.620863949388048</v>
+        <v>0.664768666809813</v>
       </c>
       <c r="F16" s="29">
         <f>F15/F7</f>
-        <v>0.623637895630626</v>
+        <v>0.666599504405763</v>
       </c>
       <c r="G16" s="29">
         <f>G15/G7</f>
-        <v>0.626295174782913</v>
+        <v>0.668353340331011</v>
       </c>
     </row>
     <row r="18" ht="18" customHeight="1" s="12">
@@ -5955,23 +5955,23 @@
       </c>
       <c r="C22" s="53">
         <f>C15*C21</f>
-        <v>1.23634409672489</v>
+        <v>1.32866943919872</v>
       </c>
       <c r="D22" s="53">
         <f>D15*D21</f>
-        <v>1.16216463278362</v>
+        <v>1.24658643421471</v>
       </c>
       <c r="E22" s="53">
         <f>E15*E21</f>
-        <v>1.09162521759919</v>
+        <v>1.16882006319524</v>
       </c>
       <c r="F22" s="53">
         <f>F15*F21</f>
-        <v>1.02464624332743</v>
+        <v>1.09523279899886</v>
       </c>
       <c r="G22" s="53">
         <f>G15*G21</f>
-        <v>0.961135056568267</v>
+        <v>1.02567902712854</v>
       </c>
     </row>
     <row r="24" ht="18" customHeight="1" s="12">
@@ -6145,11 +6145,11 @@
       </c>
       <c r="C40" s="30">
         <f>SUM(C22:G22)</f>
-        <v>5.4759152470034</v>
+        <v>5.86498776273608</v>
       </c>
       <c r="D40" s="30">
         <f>C40</f>
-        <v>5.4759152470034</v>
+        <v>5.86498776273608</v>
       </c>
     </row>
     <row r="41">
@@ -6160,7 +6160,7 @@
       </c>
       <c r="C41" s="30">
         <f>G15</f>
-        <v>1.82944303652426</v>
+        <v>1.95229727712674</v>
       </c>
       <c r="D41" s="30">
         <f>'Income Statement'!L11</f>
@@ -6190,7 +6190,7 @@
       </c>
       <c r="C43" s="30">
         <f>C41*(1+C42)/(C36-C42)</f>
-        <v>14.562377226131</v>
+        <v>15.5402976968784</v>
       </c>
       <c r="D43" s="30">
         <f>D41*D42</f>
@@ -6220,7 +6220,7 @@
       </c>
       <c r="C45" s="30">
         <f>C43*C44</f>
-        <v>7.12259774125004</v>
+        <v>7.60090798056786</v>
       </c>
       <c r="D45" s="30">
         <f>D43*D44</f>
@@ -6235,11 +6235,11 @@
       </c>
       <c r="C46" s="59">
         <f>C40+C45</f>
-        <v>12.5985129882534</v>
+        <v>13.4658957433039</v>
       </c>
       <c r="D46" s="59">
         <f>D40+D45</f>
-        <v>13.3338542968362</v>
+        <v>13.7229268125689</v>
       </c>
     </row>
     <row r="47">
@@ -6250,11 +6250,11 @@
       </c>
       <c r="C47" s="29">
         <f>C45/C46</f>
-        <v>0.565352256086968</v>
+        <v>0.564456173243989</v>
       </c>
       <c r="D47" s="29">
         <f>D45/D46</f>
-        <v>0.589322402577724</v>
+        <v>0.572613929751174</v>
       </c>
     </row>
     <row r="48">
@@ -6265,11 +6265,11 @@
       </c>
       <c r="C48" s="56">
         <f>C46/Assumptions!C46</f>
-        <v>6.29925649412672</v>
+        <v>6.73294787165197</v>
       </c>
       <c r="D48" s="56">
         <f>D46/Assumptions!C46</f>
-        <v>6.66692714841812</v>
+        <v>6.86146340628446</v>
       </c>
     </row>
     <row r="49">
@@ -6280,11 +6280,11 @@
       </c>
       <c r="C49" s="56">
         <f>C43/'Income Statement'!L11</f>
-        <v>4.98531323906216</v>
+        <v>5.32009648178837</v>
       </c>
       <c r="D49" s="65">
         <f>(D43*C36-G15)/(D43+G15)</f>
-        <v>0.0358182137746673</v>
+        <v>0.0287556135134551</v>
       </c>
     </row>
     <row r="50">
@@ -6310,11 +6310,11 @@
       </c>
       <c r="C51" s="46">
         <f>C46+C50</f>
-        <v>12.5985129882534</v>
+        <v>13.4658957433039</v>
       </c>
       <c r="D51" s="46">
         <f>D46+D50</f>
-        <v>13.3338542968362</v>
+        <v>13.7229268125689</v>
       </c>
     </row>
     <row r="53" ht="18" customHeight="1" s="12">
@@ -6358,23 +6358,23 @@
       </c>
       <c r="C55" s="30">
         <f>SUMPRODUCT($C$15:$G$15,1/(1+$B55)^$C$20:$G$20)+$G$15*(1+C$54)/($B55-C$54)/(1+$B55)^$G$19</f>
-        <v>14.0554485978312</v>
+        <v>15.0212073651489</v>
       </c>
       <c r="D55" s="30">
         <f>SUMPRODUCT($C$15:$G$15,1/(1+$B55)^$C$20:$G$20)+$G$15*(1+D$54)/($B55-D$54)/(1+$B55)^$G$19</f>
-        <v>14.465148437539</v>
+        <v>15.4584201482375</v>
       </c>
       <c r="E55" s="30">
         <f>SUMPRODUCT($C$15:$G$15,1/(1+$B55)^$C$20:$G$20)+$G$15*(1+E$54)/($B55-E$54)/(1+$B55)^$G$19</f>
-        <v>14.912515331406</v>
+        <v>15.9358294751945</v>
       </c>
       <c r="F55" s="30">
         <f>SUMPRODUCT($C$15:$G$15,1/(1+$B55)^$C$20:$G$20)+$G$15*(1+F$54)/($B55-F$54)/(1+$B55)^$G$19</f>
-        <v>15.4029941345778</v>
+        <v>16.4592458444409</v>
       </c>
       <c r="G55" s="30">
         <f>SUMPRODUCT($C$15:$G$15,1/(1+$B55)^$C$20:$G$20)+$G$15*(1+G$54)/($B55-G$54)/(1+$B55)^$G$19</f>
-        <v>15.9431322483282</v>
+        <v>17.035656340802</v>
       </c>
     </row>
     <row r="56">
@@ -6384,23 +6384,23 @@
       </c>
       <c r="C56" s="30">
         <f>SUMPRODUCT($C$15:$G$15,1/(1+$B56)^$C$20:$G$20)+$G$15*(1+C$54)/($B56-C$54)/(1+$B56)^$G$19</f>
-        <v>12.9575712734512</v>
+        <v>13.8493311170763</v>
       </c>
       <c r="D56" s="30">
         <f>SUMPRODUCT($C$15:$G$15,1/(1+$B56)^$C$20:$G$20)+$G$15*(1+D$54)/($B56-D$54)/(1+$B56)^$G$19</f>
-        <v>13.2929337782018</v>
+        <v>14.2072145230111</v>
       </c>
       <c r="E56" s="30">
         <f>SUMPRODUCT($C$15:$G$15,1/(1+$B56)^$C$20:$G$20)+$G$15*(1+E$54)/($B56-E$54)/(1+$B56)^$G$19</f>
-        <v>13.6565328775745</v>
+        <v>14.5952307211102</v>
       </c>
       <c r="F56" s="30">
         <f>SUMPRODUCT($C$15:$G$15,1/(1+$B56)^$C$20:$G$20)+$G$15*(1+F$54)/($B56-F$54)/(1+$B56)^$G$19</f>
-        <v>14.0520914648884</v>
+        <v>15.0173526115104</v>
       </c>
       <c r="G56" s="30">
         <f>SUMPRODUCT($C$15:$G$15,1/(1+$B56)^$C$20:$G$20)+$G$15*(1+G$54)/($B56-G$54)/(1+$B56)^$G$19</f>
-        <v>14.4840169854727</v>
+        <v>15.4782836166978</v>
       </c>
     </row>
     <row r="57">
@@ -6410,23 +6410,23 @@
       </c>
       <c r="C57" s="30">
         <f>SUMPRODUCT($C$15:$G$15,1/(1+$B57)^$C$20:$G$20)+$G$15*(1+C$54)/($B57-C$54)/(1+$B57)^$G$19</f>
-        <v>12.0207607351178</v>
+        <v>12.849345171282</v>
       </c>
       <c r="D57" s="30">
         <f>SUMPRODUCT($C$15:$G$15,1/(1+$B57)^$C$20:$G$20)+$G$15*(1+D$54)/($B57-D$54)/(1+$B57)^$G$19</f>
-        <v>12.2988392678318</v>
+        <v>13.1460977628666</v>
       </c>
       <c r="E57" s="59">
         <f>SUMPRODUCT($C$15:$G$15,1/(1+$B57)^$C$20:$G$20)+$G$15*(1+E$54)/($B57-E$54)/(1+$B57)^$G$19</f>
-        <v>12.5985129882534</v>
+        <v>13.4658957433039</v>
       </c>
       <c r="F57" s="30">
         <f>SUMPRODUCT($C$15:$G$15,1/(1+$B57)^$C$20:$G$20)+$G$15*(1+F$54)/($B57-F$54)/(1+$B57)^$G$19</f>
-        <v>12.9223990983471</v>
+        <v>13.8115320698858</v>
       </c>
       <c r="G57" s="30">
         <f>SUMPRODUCT($C$15:$G$15,1/(1+$B57)^$C$20:$G$20)+$G$15*(1+G$54)/($B57-G$54)/(1+$B57)^$G$19</f>
-        <v>13.2735555223991</v>
+        <v>14.1862700184501</v>
       </c>
     </row>
     <row r="58">
@@ -6436,23 +6436,23 @@
       </c>
       <c r="C58" s="30">
         <f>SUMPRODUCT($C$15:$G$15,1/(1+$B58)^$C$20:$G$20)+$G$15*(1+C$54)/($B58-C$54)/(1+$B58)^$G$19</f>
-        <v>11.2123392122309</v>
+        <v>11.9863770449078</v>
       </c>
       <c r="D58" s="30">
         <f>SUMPRODUCT($C$15:$G$15,1/(1+$B58)^$C$20:$G$20)+$G$15*(1+D$54)/($B58-D$54)/(1+$B58)^$G$19</f>
-        <v>11.4454948495028</v>
+        <v>12.2351899932778</v>
       </c>
       <c r="E58" s="30">
         <f>SUMPRODUCT($C$15:$G$15,1/(1+$B58)^$C$20:$G$20)+$G$15*(1+E$54)/($B58-E$54)/(1+$B58)^$G$19</f>
-        <v>11.6954522261628</v>
+        <v>12.5019329834166</v>
       </c>
       <c r="F58" s="30">
         <f>SUMPRODUCT($C$15:$G$15,1/(1+$B58)^$C$20:$G$20)+$G$15*(1+F$54)/($B58-F$54)/(1+$B58)^$G$19</f>
-        <v>11.9640953853138</v>
+        <v>12.7886165792752</v>
       </c>
       <c r="G58" s="30">
         <f>SUMPRODUCT($C$15:$G$15,1/(1+$B58)^$C$20:$G$20)+$G$15*(1+G$54)/($B58-G$54)/(1+$B58)^$G$19</f>
-        <v>12.2536009943334</v>
+        <v>13.0975636199416</v>
       </c>
     </row>
     <row r="59">
@@ -6462,23 +6462,23 @@
       </c>
       <c r="C59" s="30">
         <f>SUMPRODUCT($C$15:$G$15,1/(1+$B59)^$C$20:$G$20)+$G$15*(1+C$54)/($B59-C$54)/(1+$B59)^$G$19</f>
-        <v>10.5078762373019</v>
+        <v>11.2343554096799</v>
       </c>
       <c r="D59" s="30">
         <f>SUMPRODUCT($C$15:$G$15,1/(1+$B59)^$C$20:$G$20)+$G$15*(1+D$54)/($B59-D$54)/(1+$B59)^$G$19</f>
-        <v>10.7052664499358</v>
+        <v>11.4450011455475</v>
       </c>
       <c r="E59" s="30">
         <f>SUMPRODUCT($C$15:$G$15,1/(1+$B59)^$C$20:$G$20)+$G$15*(1+E$54)/($B59-E$54)/(1+$B59)^$G$19</f>
-        <v>10.9159249203613</v>
+        <v>11.6698061545063</v>
       </c>
       <c r="F59" s="30">
         <f>SUMPRODUCT($C$15:$G$15,1/(1+$B59)^$C$20:$G$20)+$G$15*(1+F$54)/($B59-F$54)/(1+$B59)^$G$19</f>
-        <v>11.1412359818697</v>
+        <v>11.9102477332313</v>
       </c>
       <c r="G59" s="30">
         <f>SUMPRODUCT($C$15:$G$15,1/(1+$B59)^$C$20:$G$20)+$G$15*(1+G$54)/($B59-G$54)/(1+$B59)^$G$19</f>
-        <v>11.3827834843282</v>
+        <v>12.1680160932904</v>
       </c>
     </row>
     <row r="61" ht="18" customHeight="1" s="12">
@@ -6522,23 +6522,23 @@
       </c>
       <c r="C63" s="30">
         <f>SUMPRODUCT($C$15:$G$15,1/(1+$B63)^$C$20:$G$20)+$D$41*C$62/(1+$B63)^$G$19</f>
-        <v>12.726447191654</v>
+        <v>13.1317627689629</v>
       </c>
       <c r="D63" s="30">
         <f>SUMPRODUCT($C$15:$G$15,1/(1+$B63)^$C$20:$G$20)+$D$41*D$62/(1+$B63)^$G$19</f>
-        <v>13.5060751733681</v>
+        <v>13.9113907506771</v>
       </c>
       <c r="E63" s="30">
         <f>SUMPRODUCT($C$15:$G$15,1/(1+$B63)^$C$20:$G$20)+$D$41*E$62/(1+$B63)^$G$19</f>
-        <v>14.2857031550823</v>
+        <v>14.6910187323912</v>
       </c>
       <c r="F63" s="30">
         <f>SUMPRODUCT($C$15:$G$15,1/(1+$B63)^$C$20:$G$20)+$D$41*F$62/(1+$B63)^$G$19</f>
-        <v>15.0653311367964</v>
+        <v>15.4706467141054</v>
       </c>
       <c r="G63" s="30">
         <f>SUMPRODUCT($C$15:$G$15,1/(1+$B63)^$C$20:$G$20)+$D$41*G$62/(1+$B63)^$G$19</f>
-        <v>15.8449591185106</v>
+        <v>16.2502746958195</v>
       </c>
     </row>
     <row r="64">
@@ -6548,23 +6548,23 @@
       </c>
       <c r="C64" s="30">
         <f>SUMPRODUCT($C$15:$G$15,1/(1+$B64)^$C$20:$G$20)+$D$41*C$62/(1+$B64)^$G$19</f>
-        <v>12.3059307968511</v>
+        <v>12.7029762071139</v>
       </c>
       <c r="D64" s="30">
         <f>SUMPRODUCT($C$15:$G$15,1/(1+$B64)^$C$20:$G$20)+$D$41*D$62/(1+$B64)^$G$19</f>
-        <v>13.0520680036006</v>
+        <v>13.4491134138633</v>
       </c>
       <c r="E64" s="30">
         <f>SUMPRODUCT($C$15:$G$15,1/(1+$B64)^$C$20:$G$20)+$D$41*E$62/(1+$B64)^$G$19</f>
-        <v>13.7982052103501</v>
+        <v>14.1952506206128</v>
       </c>
       <c r="F64" s="30">
         <f>SUMPRODUCT($C$15:$G$15,1/(1+$B64)^$C$20:$G$20)+$D$41*F$62/(1+$B64)^$G$19</f>
-        <v>14.5443424170995</v>
+        <v>14.9413878273623</v>
       </c>
       <c r="G64" s="30">
         <f>SUMPRODUCT($C$15:$G$15,1/(1+$B64)^$C$20:$G$20)+$D$41*G$62/(1+$B64)^$G$19</f>
-        <v>15.290479623849</v>
+        <v>15.6875250341118</v>
       </c>
     </row>
     <row r="65">
@@ -6574,23 +6574,23 @@
       </c>
       <c r="C65" s="30">
         <f>SUMPRODUCT($C$15:$G$15,1/(1+$B65)^$C$20:$G$20)+$D$41*C$62/(1+$B65)^$G$19</f>
-        <v>11.9051381059575</v>
+        <v>12.2942106216902</v>
       </c>
       <c r="D65" s="30">
         <f>SUMPRODUCT($C$15:$G$15,1/(1+$B65)^$C$20:$G$20)+$D$41*D$62/(1+$B65)^$G$19</f>
-        <v>12.6194962013969</v>
+        <v>13.0085687171296</v>
       </c>
       <c r="E65" s="59">
         <f>SUMPRODUCT($C$15:$G$15,1/(1+$B65)^$C$20:$G$20)+$D$41*E$62/(1+$B65)^$G$19</f>
-        <v>13.3338542968362</v>
+        <v>13.7229268125689</v>
       </c>
       <c r="F65" s="30">
         <f>SUMPRODUCT($C$15:$G$15,1/(1+$B65)^$C$20:$G$20)+$D$41*F$62/(1+$B65)^$G$19</f>
-        <v>14.0482123922756</v>
+        <v>14.4372849080083</v>
       </c>
       <c r="G65" s="30">
         <f>SUMPRODUCT($C$15:$G$15,1/(1+$B65)^$C$20:$G$20)+$D$41*G$62/(1+$B65)^$G$19</f>
-        <v>14.7625704877149</v>
+        <v>15.1516430034476</v>
       </c>
     </row>
     <row r="66">
@@ -6600,23 +6600,23 @@
       </c>
       <c r="C66" s="30">
         <f>SUMPRODUCT($C$15:$G$15,1/(1+$B66)^$C$20:$G$20)+$D$41*C$62/(1+$B66)^$G$19</f>
-        <v>11.5229544750503</v>
+        <v>11.9043374051759</v>
       </c>
       <c r="D66" s="30">
         <f>SUMPRODUCT($C$15:$G$15,1/(1+$B66)^$C$20:$G$20)+$D$41*D$62/(1+$B66)^$G$19</f>
-        <v>12.2071439265797</v>
+        <v>12.5885268567052</v>
       </c>
       <c r="E66" s="30">
         <f>SUMPRODUCT($C$15:$G$15,1/(1+$B66)^$C$20:$G$20)+$D$41*E$62/(1+$B66)^$G$19</f>
-        <v>12.891333378109</v>
+        <v>13.2727163082346</v>
       </c>
       <c r="F66" s="30">
         <f>SUMPRODUCT($C$15:$G$15,1/(1+$B66)^$C$20:$G$20)+$D$41*F$62/(1+$B66)^$G$19</f>
-        <v>13.5755228296384</v>
+        <v>13.956905759764</v>
       </c>
       <c r="G66" s="30">
         <f>SUMPRODUCT($C$15:$G$15,1/(1+$B66)^$C$20:$G$20)+$D$41*G$62/(1+$B66)^$G$19</f>
-        <v>14.2597122811678</v>
+        <v>14.6410952112933</v>
       </c>
     </row>
     <row r="67">
@@ -6626,23 +6626,23 @@
       </c>
       <c r="C67" s="30">
         <f>SUMPRODUCT($C$15:$G$15,1/(1+$B67)^$C$20:$G$20)+$D$41*C$62/(1+$B67)^$G$19</f>
-        <v>11.1583378590632</v>
+        <v>11.5323013392616</v>
       </c>
       <c r="D67" s="30">
         <f>SUMPRODUCT($C$15:$G$15,1/(1+$B67)^$C$20:$G$20)+$D$41*D$62/(1+$B67)^$G$19</f>
-        <v>11.8138747179835</v>
+        <v>12.1878381981818</v>
       </c>
       <c r="E67" s="30">
         <f>SUMPRODUCT($C$15:$G$15,1/(1+$B67)^$C$20:$G$20)+$D$41*E$62/(1+$B67)^$G$19</f>
-        <v>12.4694115769037</v>
+        <v>12.843375057102</v>
       </c>
       <c r="F67" s="30">
         <f>SUMPRODUCT($C$15:$G$15,1/(1+$B67)^$C$20:$G$20)+$D$41*F$62/(1+$B67)^$G$19</f>
-        <v>13.1249484358239</v>
+        <v>13.4989119160222</v>
       </c>
       <c r="G67" s="30">
         <f>SUMPRODUCT($C$15:$G$15,1/(1+$B67)^$C$20:$G$20)+$D$41*G$62/(1+$B67)^$G$19</f>
-        <v>13.7804852947441</v>
+        <v>14.1544487749424</v>
       </c>
     </row>
     <row r="69" ht="40" customHeight="1" s="12">

</xml_diff>